<commit_message>
docs and rebound stop adjustmetns
</commit_message>
<xml_diff>
--- a/docs/damping_curve_RAx0.xlsx
+++ b/docs/damping_curve_RAx0.xlsx
@@ -6806,9 +6806,7 @@
       <c r="D11" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="E11" s="49" t="s">
-        <v>111</v>
-      </c>
+      <c r="E11" s="48"/>
       <c r="F11" s="49" t="s">
         <v>111</v>
       </c>

</xml_diff>

<commit_message>
Fix hydraulic stops and others
</commit_message>
<xml_diff>
--- a/docs/damping_curve_RAx0.xlsx
+++ b/docs/damping_curve_RAx0.xlsx
@@ -6752,8 +6752,8 @@
       <c r="D8" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="E8" s="29">
-        <v>20</v>
+      <c s="29" r="E8" t="n">
+        <v>10</v>
       </c>
       <c r="F8" s="29">
         <v>20</v>
@@ -7097,8 +7097,8 @@
       <c r="B8" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="61">
-        <v>-10</v>
+      <c s="61" r="C8" t="n">
+        <v>-5</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -7228,9 +7228,9 @@
       <c r="B14" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="69">
-        <f>Parameters!D24</f>
-        <v>20</v>
+      <c s="69" r="C14" t="n">
+        <f>IF(C6="RA60",Parameters!D27,Parameters!D24)</f>
+        <v>10</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -7832,7 +7832,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="whole" sqref="C8" xr:uid="{00000000-0002-0000-0500-000003000000}">
-      <formula1>-20</formula1>
+      <formula1>-C14</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="whole" sqref="C9" xr:uid="{00000000-0002-0000-0500-000004000000}">
@@ -11637,10 +11637,8 @@
         <v>24</v>
       </c>
       <c r="E23" s="1"/>
-      <c r="F23" s="90" t="inlineStr">
-        <is>
-          <t>Sweep 使用 40 格 R；计算器按型号换算。</t>
-        </is>
+      <c s="90" r="F23" t="str">
+        <v>Sweep 使用 8 系 C、40 格 R。</v>
       </c>
       <c r="G23" s="91"/>
       <c r="H23" s="91"/>
@@ -11654,8 +11652,8 @@
     </row>
     <row r="24" spans="1:15" ht="29" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="62" t="s">
-        <v>67</v>
+      <c s="62" r="B24" t="str">
+        <v>HSC · 8 系</v>
       </c>
       <c r="C24" s="73"/>
       <c r="D24" s="69">
@@ -11719,11 +11717,15 @@
       <c r="N26" s="82"/>
       <c r="O26" s="1"/>
     </row>
-    <row r="27" spans="1:15" ht="12" customHeight="1">
+    <row r="27" spans="1:15" ht="29" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
+      <c s="62" r="B27" t="str">
+        <v>HSC · 6 系</v>
+      </c>
+      <c s="73" r="C27"/>
+      <c s="69" r="D27" t="n">
+        <v>10</v>
+      </c>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
@@ -11979,7 +11981,8 @@
       <c r="O41" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
+    <mergeCell ref="B27:C27"/>
     <mergeCell ref="B2:N2"/>
     <mergeCell ref="B3:N3"/>
     <mergeCell ref="D5:H5"/>
@@ -19058,9 +19061,9 @@
         <f>Calculator!C7</f>
         <v>-12</v>
       </c>
-      <c r="D165" s="117">
+      <c s="117" r="D165" t="n">
         <f>Calculator!C8</f>
-        <v>-10</v>
+        <v>-5</v>
       </c>
       <c r="E165" s="117">
         <f>Calculator!C9</f>
@@ -19114,8 +19117,8 @@
         <f>MIN(4,MAX(1,INT((1+C165/Parameters!$D$23)*4)+1))</f>
         <v>3</v>
       </c>
-      <c r="R165" s="117">
-        <f>MIN(4,MAX(1,INT((1+D165/Parameters!$D$24)*4)+1))</f>
+      <c s="117" r="R165" t="n">
+        <f>MIN(4,MAX(1,INT((1+D165/Calculator!$C$14)*4)+1))</f>
         <v>3</v>
       </c>
       <c r="S165" s="117">
@@ -19126,8 +19129,8 @@
         <f>MAX(0,MIN(1,(1+C165/Parameters!$D$23)*4-(Q165-1)))</f>
         <v>0</v>
       </c>
-      <c r="U165" s="117">
-        <f>MAX(0,MIN(1,(1+D165/Parameters!$D$24)*4-(R165-1)))</f>
+      <c s="117" r="U165" t="n">
+        <f>MAX(0,MIN(1,(1+D165/Calculator!$C$14)*4-(R165-1)))</f>
         <v>0</v>
       </c>
       <c r="V165" s="117">

</xml_diff>

<commit_message>
Update gravel setups, remove RA80/2 HRS and hide WRC Kit
</commit_message>
<xml_diff>
--- a/docs/damping_curve_RAx0.xlsx
+++ b/docs/damping_curve_RAx0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mods\unpacked\un1corn_qlourie_astral_r\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26A79284-0296-47CC-94EA-B1A0D79C5356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E71426E-0C2C-43A5-9E07-AAA127F4B1D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalog" sheetId="8" r:id="rId1"/>
@@ -1880,11 +1880,11 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1899,13 +1899,13 @@
     <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1920,28 +1920,28 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="8" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="8" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="8" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1950,7 +1950,7 @@
     <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2082,26 +2082,53 @@
     <xf numFmtId="0" fontId="82" fillId="71" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="43" fillId="32" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="33" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="23" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="24" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="26" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="28" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2109,41 +2136,23 @@
     <xf numFmtId="0" fontId="23" fillId="12" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="28" fillId="17" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="29" fillId="18" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="23" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="46" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="24" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="26" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="28" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="58" fillId="47" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="32" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="33" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="45" fillId="34" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2159,18 +2168,6 @@
     </xf>
     <xf numFmtId="0" fontId="56" fillId="45" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="57" fillId="46" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="58" fillId="47" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="59" fillId="48" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -6585,14 +6582,14 @@
     </row>
     <row r="2" spans="1:8" ht="35" customHeight="1">
       <c r="A2" s="6"/>
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="72" t="s">
         <v>84</v>
       </c>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
       <c r="H2" s="6"/>
     </row>
     <row r="3" spans="1:8" ht="25" customHeight="1">
@@ -6643,7 +6640,7 @@
     </row>
     <row r="6" spans="1:8" ht="31" customHeight="1">
       <c r="A6" s="6"/>
-      <c r="B6" s="70" t="s">
+      <c r="B6" s="74" t="s">
         <v>81</v>
       </c>
       <c r="C6" s="6"/>
@@ -6663,7 +6660,7 @@
     </row>
     <row r="7" spans="1:8" ht="31" customHeight="1">
       <c r="A7" s="6"/>
-      <c r="B7" s="70"/>
+      <c r="B7" s="74"/>
       <c r="C7" s="6"/>
       <c r="D7" s="19" t="s">
         <v>77</v>
@@ -6746,9 +6743,7 @@
       <c r="F11" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="G11" s="22" t="s">
-        <v>83</v>
-      </c>
+      <c r="G11" s="21"/>
       <c r="H11" s="6"/>
     </row>
     <row r="12" spans="1:8" ht="31" customHeight="1">
@@ -6797,40 +6792,40 @@
       <c r="A15" s="6"/>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
-      <c r="D15" s="67"/>
-      <c r="E15" s="67"/>
-      <c r="F15" s="67"/>
-      <c r="G15" s="67"/>
+      <c r="D15" s="71"/>
+      <c r="E15" s="71"/>
+      <c r="F15" s="71"/>
+      <c r="G15" s="71"/>
       <c r="H15" s="6"/>
     </row>
     <row r="16" spans="1:8" ht="22" customHeight="1">
       <c r="A16" s="6"/>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
-      <c r="D16" s="67"/>
-      <c r="E16" s="67"/>
-      <c r="F16" s="67"/>
-      <c r="G16" s="67"/>
+      <c r="D16" s="71"/>
+      <c r="E16" s="71"/>
+      <c r="F16" s="71"/>
+      <c r="G16" s="71"/>
       <c r="H16" s="6"/>
     </row>
     <row r="17" spans="1:8" ht="22" customHeight="1">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="67"/>
-      <c r="F17" s="67"/>
-      <c r="G17" s="67"/>
+      <c r="D17" s="69"/>
+      <c r="E17" s="71"/>
+      <c r="F17" s="71"/>
+      <c r="G17" s="71"/>
       <c r="H17" s="6"/>
     </row>
     <row r="18" spans="1:8" ht="22" customHeight="1">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
-      <c r="D18" s="67"/>
-      <c r="E18" s="67"/>
-      <c r="F18" s="67"/>
-      <c r="G18" s="67"/>
+      <c r="D18" s="71"/>
+      <c r="E18" s="71"/>
+      <c r="F18" s="71"/>
+      <c r="G18" s="71"/>
       <c r="H18" s="6"/>
     </row>
     <row r="19" spans="1:8" ht="25" customHeight="1">
@@ -6912,20 +6907,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="71" t="s">
+      <c r="B2" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
-      <c r="L2" s="72"/>
-      <c r="M2" s="72"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="67"/>
+      <c r="M2" s="67"/>
       <c r="N2" s="24"/>
       <c r="O2" s="1"/>
     </row>
@@ -6955,15 +6950,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="73"/>
-      <c r="I4" s="73"/>
-      <c r="J4" s="73"/>
-      <c r="K4" s="73"/>
-      <c r="L4" s="73"/>
-      <c r="M4" s="73"/>
+      <c r="E4" s="68"/>
+      <c r="F4" s="68"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="68"/>
+      <c r="I4" s="68"/>
+      <c r="J4" s="68"/>
+      <c r="K4" s="68"/>
+      <c r="L4" s="68"/>
+      <c r="M4" s="68"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -6994,13 +6989,13 @@
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
-      <c r="F6" s="74" t="s">
+      <c r="F6" s="83" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="75"/>
-      <c r="H6" s="75"/>
-      <c r="I6" s="75"/>
-      <c r="J6" s="75"/>
+      <c r="G6" s="84"/>
+      <c r="H6" s="84"/>
+      <c r="I6" s="84"/>
+      <c r="J6" s="84"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
@@ -7038,16 +7033,16 @@
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
-      <c r="F8" s="76" t="s">
+      <c r="F8" s="82" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="77"/>
-      <c r="H8" s="77"/>
-      <c r="I8" s="78">
+      <c r="G8" s="79"/>
+      <c r="H8" s="79"/>
+      <c r="I8" s="85">
         <f>IF(C18="OK",Samples!F165*MIN(C10,Samples!G165)+Samples!I165*MAX(0,C10-Samples!G165)+Samples!J165*MAX(0,C10-Samples!K165),"检查输入")</f>
         <v>1736.47</v>
       </c>
-      <c r="J8" s="79"/>
+      <c r="J8" s="86"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
@@ -7085,16 +7080,16 @@
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="76" t="s">
+      <c r="F10" s="82" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="77"/>
-      <c r="H10" s="77"/>
-      <c r="I10" s="78">
+      <c r="G10" s="79"/>
+      <c r="H10" s="79"/>
+      <c r="I10" s="85">
         <f>IF(C18="OK",Samples!M165*MIN(C10,Samples!N165)+Samples!P165*MAX(0,C10-Samples!N165),"检查输入")</f>
         <v>1519.2</v>
       </c>
-      <c r="J10" s="79"/>
+      <c r="J10" s="86"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
@@ -7146,13 +7141,13 @@
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="F13" s="74" t="s">
+      <c r="F13" s="83" t="s">
         <v>47</v>
       </c>
-      <c r="G13" s="75"/>
-      <c r="H13" s="75"/>
-      <c r="I13" s="75"/>
-      <c r="J13" s="75"/>
+      <c r="G13" s="84"/>
+      <c r="H13" s="84"/>
+      <c r="I13" s="84"/>
+      <c r="J13" s="84"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
@@ -7170,11 +7165,11 @@
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
-      <c r="F14" s="80" t="s">
+      <c r="F14" s="77" t="s">
         <v>10</v>
       </c>
-      <c r="G14" s="81"/>
-      <c r="H14" s="81"/>
+      <c r="G14" s="78"/>
+      <c r="H14" s="78"/>
       <c r="I14" s="34">
         <f>Samples!F165</f>
         <v>3650</v>
@@ -7199,11 +7194,11 @@
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
-      <c r="F15" s="77" t="s">
+      <c r="F15" s="79" t="s">
         <v>26</v>
       </c>
-      <c r="G15" s="82"/>
-      <c r="H15" s="82"/>
+      <c r="G15" s="80"/>
+      <c r="H15" s="80"/>
       <c r="I15" s="35">
         <f>Samples!I165</f>
         <v>3431</v>
@@ -7223,11 +7218,11 @@
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="83" t="s">
+      <c r="F16" s="81" t="s">
         <v>48</v>
       </c>
-      <c r="G16" s="81"/>
-      <c r="H16" s="81"/>
+      <c r="G16" s="78"/>
+      <c r="H16" s="78"/>
       <c r="I16" s="34">
         <f>Samples!J165</f>
         <v>1750</v>
@@ -7247,11 +7242,11 @@
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
-      <c r="F17" s="76" t="s">
+      <c r="F17" s="82" t="s">
         <v>27</v>
       </c>
-      <c r="G17" s="82"/>
-      <c r="H17" s="82"/>
+      <c r="G17" s="80"/>
+      <c r="H17" s="80"/>
       <c r="I17" s="35">
         <f>Samples!L165</f>
         <v>5181</v>
@@ -7293,11 +7288,11 @@
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
-      <c r="F19" s="80" t="s">
+      <c r="F19" s="77" t="s">
         <v>15</v>
       </c>
-      <c r="G19" s="81"/>
-      <c r="H19" s="81"/>
+      <c r="G19" s="78"/>
+      <c r="H19" s="78"/>
       <c r="I19" s="34">
         <f>Samples!M165</f>
         <v>3600</v>
@@ -7317,11 +7312,11 @@
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
-      <c r="F20" s="77" t="s">
+      <c r="F20" s="79" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="82"/>
-      <c r="H20" s="82"/>
+      <c r="G20" s="80"/>
+      <c r="H20" s="80"/>
       <c r="I20" s="35">
         <f>Samples!P165</f>
         <v>3096</v>
@@ -7358,11 +7353,11 @@
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="83" t="s">
+      <c r="F22" s="81" t="s">
         <v>44</v>
       </c>
-      <c r="G22" s="81"/>
-      <c r="H22" s="81"/>
+      <c r="G22" s="78"/>
+      <c r="H22" s="78"/>
       <c r="I22" s="37">
         <f>Samples!G165</f>
         <v>0.08</v>
@@ -7382,11 +7377,11 @@
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="76" t="s">
+      <c r="F23" s="82" t="s">
         <v>45</v>
       </c>
-      <c r="G23" s="82"/>
-      <c r="H23" s="82"/>
+      <c r="G23" s="80"/>
+      <c r="H23" s="80"/>
       <c r="I23" s="38">
         <f>Samples!K165</f>
         <v>0.35</v>
@@ -7406,11 +7401,11 @@
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="80" t="s">
+      <c r="F24" s="77" t="s">
         <v>16</v>
       </c>
-      <c r="G24" s="81"/>
-      <c r="H24" s="81"/>
+      <c r="G24" s="78"/>
+      <c r="H24" s="78"/>
       <c r="I24" s="37">
         <f>Samples!N165</f>
         <v>0.25</v>
@@ -7460,20 +7455,20 @@
     </row>
     <row r="27" spans="1:15" ht="23.15" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="84" t="s">
+      <c r="B27" s="75" t="s">
         <v>87</v>
       </c>
-      <c r="C27" s="85"/>
-      <c r="D27" s="85"/>
-      <c r="E27" s="85"/>
-      <c r="F27" s="85"/>
-      <c r="G27" s="85"/>
-      <c r="H27" s="85"/>
-      <c r="I27" s="85"/>
-      <c r="J27" s="85"/>
-      <c r="K27" s="85"/>
-      <c r="L27" s="85"/>
-      <c r="M27" s="85"/>
+      <c r="C27" s="76"/>
+      <c r="D27" s="76"/>
+      <c r="E27" s="76"/>
+      <c r="F27" s="76"/>
+      <c r="G27" s="76"/>
+      <c r="H27" s="76"/>
+      <c r="I27" s="76"/>
+      <c r="J27" s="76"/>
+      <c r="K27" s="76"/>
+      <c r="L27" s="76"/>
+      <c r="M27" s="76"/>
       <c r="N27" s="1"/>
       <c r="O27" s="1"/>
     </row>
@@ -7734,17 +7729,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B27:M27"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="F24:H24"/>
-    <mergeCell ref="F13:J13"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="F16:H16"/>
-    <mergeCell ref="F17:H17"/>
     <mergeCell ref="B2:M2"/>
     <mergeCell ref="E4:M4"/>
     <mergeCell ref="F6:J6"/>
@@ -7752,6 +7736,17 @@
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="I10:J10"/>
+    <mergeCell ref="F13:J13"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="B27:M27"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="F24:H24"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <dataValidations count="5">
@@ -7808,20 +7803,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="71" t="s">
+      <c r="B2" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
-      <c r="L2" s="72"/>
-      <c r="M2" s="72"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="67"/>
+      <c r="M2" s="67"/>
       <c r="N2" s="24"/>
       <c r="O2" s="1"/>
     </row>
@@ -7851,15 +7846,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="73"/>
-      <c r="I4" s="73"/>
-      <c r="J4" s="73"/>
-      <c r="K4" s="73"/>
-      <c r="L4" s="73"/>
-      <c r="M4" s="73"/>
+      <c r="E4" s="68"/>
+      <c r="F4" s="68"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="68"/>
+      <c r="I4" s="68"/>
+      <c r="J4" s="68"/>
+      <c r="K4" s="68"/>
+      <c r="L4" s="68"/>
+      <c r="M4" s="68"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -7889,15 +7884,15 @@
         <v>-10</v>
       </c>
       <c r="D6" s="1"/>
-      <c r="E6" s="86"/>
-      <c r="F6" s="86"/>
-      <c r="G6" s="86"/>
-      <c r="H6" s="86"/>
-      <c r="I6" s="86"/>
-      <c r="J6" s="86"/>
-      <c r="K6" s="86"/>
-      <c r="L6" s="86"/>
-      <c r="M6" s="86"/>
+      <c r="E6" s="69"/>
+      <c r="F6" s="69"/>
+      <c r="G6" s="69"/>
+      <c r="H6" s="69"/>
+      <c r="I6" s="69"/>
+      <c r="J6" s="69"/>
+      <c r="K6" s="69"/>
+      <c r="L6" s="69"/>
+      <c r="M6" s="69"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -8481,18 +8476,18 @@
     </row>
     <row r="41" spans="1:15" ht="23.15" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="87"/>
-      <c r="C41" s="87"/>
-      <c r="D41" s="87"/>
-      <c r="E41" s="87"/>
-      <c r="F41" s="87"/>
-      <c r="G41" s="87"/>
-      <c r="H41" s="87"/>
-      <c r="I41" s="87"/>
-      <c r="J41" s="87"/>
-      <c r="K41" s="87"/>
-      <c r="L41" s="87"/>
-      <c r="M41" s="87"/>
+      <c r="B41" s="70"/>
+      <c r="C41" s="70"/>
+      <c r="D41" s="70"/>
+      <c r="E41" s="70"/>
+      <c r="F41" s="70"/>
+      <c r="G41" s="70"/>
+      <c r="H41" s="70"/>
+      <c r="I41" s="70"/>
+      <c r="J41" s="70"/>
+      <c r="K41" s="70"/>
+      <c r="L41" s="70"/>
+      <c r="M41" s="70"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -8566,20 +8561,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="71" t="s">
+      <c r="B2" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
-      <c r="L2" s="72"/>
-      <c r="M2" s="72"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="67"/>
+      <c r="M2" s="67"/>
       <c r="N2" s="24"/>
       <c r="O2" s="1"/>
     </row>
@@ -8609,15 +8604,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="73"/>
-      <c r="I4" s="73"/>
-      <c r="J4" s="73"/>
-      <c r="K4" s="73"/>
-      <c r="L4" s="73"/>
-      <c r="M4" s="73"/>
+      <c r="E4" s="68"/>
+      <c r="F4" s="68"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="68"/>
+      <c r="I4" s="68"/>
+      <c r="J4" s="68"/>
+      <c r="K4" s="68"/>
+      <c r="L4" s="68"/>
+      <c r="M4" s="68"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -8647,15 +8642,15 @@
         <v>-12</v>
       </c>
       <c r="D6" s="1"/>
-      <c r="E6" s="86"/>
-      <c r="F6" s="86"/>
-      <c r="G6" s="86"/>
-      <c r="H6" s="86"/>
-      <c r="I6" s="86"/>
-      <c r="J6" s="86"/>
-      <c r="K6" s="86"/>
-      <c r="L6" s="86"/>
-      <c r="M6" s="86"/>
+      <c r="E6" s="69"/>
+      <c r="F6" s="69"/>
+      <c r="G6" s="69"/>
+      <c r="H6" s="69"/>
+      <c r="I6" s="69"/>
+      <c r="J6" s="69"/>
+      <c r="K6" s="69"/>
+      <c r="L6" s="69"/>
+      <c r="M6" s="69"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -9239,18 +9234,18 @@
     </row>
     <row r="41" spans="1:15" ht="23.15" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="87"/>
-      <c r="C41" s="87"/>
-      <c r="D41" s="87"/>
-      <c r="E41" s="87"/>
-      <c r="F41" s="87"/>
-      <c r="G41" s="87"/>
-      <c r="H41" s="87"/>
-      <c r="I41" s="87"/>
-      <c r="J41" s="87"/>
-      <c r="K41" s="87"/>
-      <c r="L41" s="87"/>
-      <c r="M41" s="87"/>
+      <c r="B41" s="70"/>
+      <c r="C41" s="70"/>
+      <c r="D41" s="70"/>
+      <c r="E41" s="70"/>
+      <c r="F41" s="70"/>
+      <c r="G41" s="70"/>
+      <c r="H41" s="70"/>
+      <c r="I41" s="70"/>
+      <c r="J41" s="70"/>
+      <c r="K41" s="70"/>
+      <c r="L41" s="70"/>
+      <c r="M41" s="70"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -9324,20 +9319,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="71" t="s">
+      <c r="B2" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
-      <c r="L2" s="72"/>
-      <c r="M2" s="72"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="67"/>
+      <c r="M2" s="67"/>
       <c r="N2" s="24"/>
       <c r="O2" s="1"/>
     </row>
@@ -9367,15 +9362,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="73"/>
-      <c r="I4" s="73"/>
-      <c r="J4" s="73"/>
-      <c r="K4" s="73"/>
-      <c r="L4" s="73"/>
-      <c r="M4" s="73"/>
+      <c r="E4" s="68"/>
+      <c r="F4" s="68"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="68"/>
+      <c r="I4" s="68"/>
+      <c r="J4" s="68"/>
+      <c r="K4" s="68"/>
+      <c r="L4" s="68"/>
+      <c r="M4" s="68"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -9398,18 +9393,18 @@
     </row>
     <row r="6" spans="1:15" ht="28" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="86"/>
-      <c r="C6" s="86"/>
-      <c r="D6" s="86"/>
-      <c r="E6" s="86"/>
-      <c r="F6" s="86"/>
-      <c r="G6" s="86"/>
-      <c r="H6" s="86"/>
-      <c r="I6" s="86"/>
-      <c r="J6" s="86"/>
-      <c r="K6" s="86"/>
-      <c r="L6" s="86"/>
-      <c r="M6" s="86"/>
+      <c r="B6" s="69"/>
+      <c r="C6" s="69"/>
+      <c r="D6" s="69"/>
+      <c r="E6" s="69"/>
+      <c r="F6" s="69"/>
+      <c r="G6" s="69"/>
+      <c r="H6" s="69"/>
+      <c r="I6" s="69"/>
+      <c r="J6" s="69"/>
+      <c r="K6" s="69"/>
+      <c r="L6" s="69"/>
+      <c r="M6" s="69"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -9993,18 +9988,18 @@
     </row>
     <row r="41" spans="1:15" ht="23.15" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="87"/>
-      <c r="C41" s="87"/>
-      <c r="D41" s="87"/>
-      <c r="E41" s="87"/>
-      <c r="F41" s="87"/>
-      <c r="G41" s="87"/>
-      <c r="H41" s="87"/>
-      <c r="I41" s="87"/>
-      <c r="J41" s="87"/>
-      <c r="K41" s="87"/>
-      <c r="L41" s="87"/>
-      <c r="M41" s="87"/>
+      <c r="B41" s="70"/>
+      <c r="C41" s="70"/>
+      <c r="D41" s="70"/>
+      <c r="E41" s="70"/>
+      <c r="F41" s="70"/>
+      <c r="G41" s="70"/>
+      <c r="H41" s="70"/>
+      <c r="I41" s="70"/>
+      <c r="J41" s="70"/>
+      <c r="K41" s="70"/>
+      <c r="L41" s="70"/>
+      <c r="M41" s="70"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -10074,20 +10069,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="71" t="s">
+      <c r="B2" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
-      <c r="L2" s="72"/>
-      <c r="M2" s="72"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="67"/>
+      <c r="M2" s="67"/>
       <c r="N2" s="24"/>
       <c r="O2" s="1"/>
     </row>
@@ -10117,15 +10112,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="73"/>
-      <c r="I4" s="73"/>
-      <c r="J4" s="73"/>
-      <c r="K4" s="73"/>
-      <c r="L4" s="73"/>
-      <c r="M4" s="73"/>
+      <c r="E4" s="68"/>
+      <c r="F4" s="68"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="68"/>
+      <c r="I4" s="68"/>
+      <c r="J4" s="68"/>
+      <c r="K4" s="68"/>
+      <c r="L4" s="68"/>
+      <c r="M4" s="68"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -10148,18 +10143,18 @@
     </row>
     <row r="6" spans="1:15" ht="28" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="86"/>
-      <c r="C6" s="86"/>
-      <c r="D6" s="86"/>
-      <c r="E6" s="86"/>
-      <c r="F6" s="86"/>
-      <c r="G6" s="86"/>
-      <c r="H6" s="86"/>
-      <c r="I6" s="86"/>
-      <c r="J6" s="86"/>
-      <c r="K6" s="86"/>
-      <c r="L6" s="86"/>
-      <c r="M6" s="86"/>
+      <c r="B6" s="69"/>
+      <c r="C6" s="69"/>
+      <c r="D6" s="69"/>
+      <c r="E6" s="69"/>
+      <c r="F6" s="69"/>
+      <c r="G6" s="69"/>
+      <c r="H6" s="69"/>
+      <c r="I6" s="69"/>
+      <c r="J6" s="69"/>
+      <c r="K6" s="69"/>
+      <c r="L6" s="69"/>
+      <c r="M6" s="69"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -10743,18 +10738,18 @@
     </row>
     <row r="41" spans="1:15" ht="23.15" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="87"/>
-      <c r="C41" s="87"/>
-      <c r="D41" s="87"/>
-      <c r="E41" s="87"/>
-      <c r="F41" s="87"/>
-      <c r="G41" s="87"/>
-      <c r="H41" s="87"/>
-      <c r="I41" s="87"/>
-      <c r="J41" s="87"/>
-      <c r="K41" s="87"/>
-      <c r="L41" s="87"/>
-      <c r="M41" s="87"/>
+      <c r="B41" s="70"/>
+      <c r="C41" s="70"/>
+      <c r="D41" s="70"/>
+      <c r="E41" s="70"/>
+      <c r="F41" s="70"/>
+      <c r="G41" s="70"/>
+      <c r="H41" s="70"/>
+      <c r="I41" s="70"/>
+      <c r="J41" s="70"/>
+      <c r="K41" s="70"/>
+      <c r="L41" s="70"/>
+      <c r="M41" s="70"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -10828,40 +10823,40 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="71" t="s">
+      <c r="B2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
-      <c r="L2" s="72"/>
-      <c r="M2" s="72"/>
-      <c r="N2" s="72"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="67"/>
+      <c r="M2" s="67"/>
+      <c r="N2" s="67"/>
       <c r="O2" s="1"/>
     </row>
     <row r="3" spans="1:15" ht="24" customHeight="1">
       <c r="A3" s="1"/>
-      <c r="B3" s="88" t="s">
+      <c r="B3" s="91" t="s">
         <v>87</v>
       </c>
-      <c r="C3" s="89"/>
-      <c r="D3" s="89"/>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="89"/>
-      <c r="H3" s="89"/>
-      <c r="I3" s="89"/>
-      <c r="J3" s="89"/>
-      <c r="K3" s="89"/>
-      <c r="L3" s="89"/>
-      <c r="M3" s="89"/>
-      <c r="N3" s="89"/>
+      <c r="C3" s="92"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="92"/>
+      <c r="F3" s="92"/>
+      <c r="G3" s="92"/>
+      <c r="H3" s="92"/>
+      <c r="I3" s="92"/>
+      <c r="J3" s="92"/>
+      <c r="K3" s="92"/>
+      <c r="L3" s="92"/>
+      <c r="M3" s="92"/>
+      <c r="N3" s="92"/>
       <c r="O3" s="1"/>
     </row>
     <row r="4" spans="1:15" ht="28" customHeight="1">
@@ -10885,21 +10880,21 @@
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
-      <c r="D5" s="75" t="s">
+      <c r="D5" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="75"/>
-      <c r="F5" s="75"/>
-      <c r="G5" s="75"/>
-      <c r="H5" s="75"/>
+      <c r="E5" s="84"/>
+      <c r="F5" s="84"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="84"/>
       <c r="I5" s="1"/>
-      <c r="J5" s="75" t="s">
+      <c r="J5" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="K5" s="75"/>
-      <c r="L5" s="75"/>
-      <c r="M5" s="75"/>
-      <c r="N5" s="75"/>
+      <c r="K5" s="84"/>
+      <c r="L5" s="84"/>
+      <c r="M5" s="84"/>
+      <c r="N5" s="84"/>
       <c r="O5" s="1"/>
     </row>
     <row r="6" spans="1:15" ht="30" customHeight="1">
@@ -11529,73 +11524,73 @@
     </row>
     <row r="22" spans="1:15" ht="32" customHeight="1">
       <c r="A22" s="1"/>
-      <c r="B22" s="74" t="s">
+      <c r="B22" s="83" t="s">
         <v>52</v>
       </c>
-      <c r="C22" s="75"/>
-      <c r="D22" s="75"/>
-      <c r="E22" s="75"/>
-      <c r="F22" s="75"/>
-      <c r="G22" s="75"/>
-      <c r="H22" s="75"/>
-      <c r="I22" s="75"/>
-      <c r="J22" s="75"/>
-      <c r="K22" s="75"/>
-      <c r="L22" s="75"/>
-      <c r="M22" s="75"/>
-      <c r="N22" s="75"/>
+      <c r="C22" s="84"/>
+      <c r="D22" s="84"/>
+      <c r="E22" s="84"/>
+      <c r="F22" s="84"/>
+      <c r="G22" s="84"/>
+      <c r="H22" s="84"/>
+      <c r="I22" s="84"/>
+      <c r="J22" s="84"/>
+      <c r="K22" s="84"/>
+      <c r="L22" s="84"/>
+      <c r="M22" s="84"/>
+      <c r="N22" s="84"/>
       <c r="O22" s="1"/>
     </row>
     <row r="23" spans="1:15" ht="29" customHeight="1">
       <c r="A23" s="1"/>
-      <c r="B23" s="83" t="s">
+      <c r="B23" s="81" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="81"/>
+      <c r="C23" s="78"/>
       <c r="D23" s="31">
         <v>24</v>
       </c>
       <c r="E23" s="1"/>
-      <c r="F23" s="90" t="s">
+      <c r="F23" s="93" t="s">
         <v>88</v>
       </c>
-      <c r="G23" s="91"/>
-      <c r="H23" s="91"/>
-      <c r="I23" s="91"/>
-      <c r="J23" s="91"/>
-      <c r="K23" s="91"/>
-      <c r="L23" s="91"/>
-      <c r="M23" s="91"/>
-      <c r="N23" s="91"/>
+      <c r="G23" s="94"/>
+      <c r="H23" s="94"/>
+      <c r="I23" s="94"/>
+      <c r="J23" s="94"/>
+      <c r="K23" s="94"/>
+      <c r="L23" s="94"/>
+      <c r="M23" s="94"/>
+      <c r="N23" s="94"/>
       <c r="O23" s="1"/>
     </row>
     <row r="24" spans="1:15" ht="29" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="76" t="s">
+      <c r="B24" s="82" t="s">
         <v>89</v>
       </c>
-      <c r="C24" s="82"/>
+      <c r="C24" s="80"/>
       <c r="D24" s="33">
         <v>20</v>
       </c>
       <c r="E24" s="1"/>
-      <c r="F24" s="91"/>
-      <c r="G24" s="91"/>
-      <c r="H24" s="91"/>
-      <c r="I24" s="91"/>
-      <c r="J24" s="91"/>
-      <c r="K24" s="91"/>
-      <c r="L24" s="91"/>
-      <c r="M24" s="91"/>
-      <c r="N24" s="91"/>
+      <c r="F24" s="94"/>
+      <c r="G24" s="94"/>
+      <c r="H24" s="94"/>
+      <c r="I24" s="94"/>
+      <c r="J24" s="94"/>
+      <c r="K24" s="94"/>
+      <c r="L24" s="94"/>
+      <c r="M24" s="94"/>
+      <c r="N24" s="94"/>
       <c r="O24" s="1"/>
     </row>
     <row r="25" spans="1:15" ht="29" customHeight="1">
       <c r="A25" s="1"/>
-      <c r="B25" s="83" t="s">
+      <c r="B25" s="81" t="s">
         <v>60</v>
       </c>
-      <c r="C25" s="81"/>
+      <c r="C25" s="78"/>
       <c r="D25" s="31">
         <v>40</v>
       </c>
@@ -11613,33 +11608,33 @@
     </row>
     <row r="26" spans="1:15" ht="29" customHeight="1">
       <c r="A26" s="1"/>
-      <c r="B26" s="77" t="s">
+      <c r="B26" s="79" t="s">
         <v>54</v>
       </c>
-      <c r="C26" s="82"/>
+      <c r="C26" s="80"/>
       <c r="D26" s="33">
         <v>60</v>
       </c>
       <c r="E26" s="1"/>
-      <c r="F26" s="92" t="s">
+      <c r="F26" s="95" t="s">
         <v>90</v>
       </c>
-      <c r="G26" s="89"/>
-      <c r="H26" s="89"/>
-      <c r="I26" s="89"/>
-      <c r="J26" s="89"/>
-      <c r="K26" s="89"/>
-      <c r="L26" s="89"/>
-      <c r="M26" s="89"/>
-      <c r="N26" s="89"/>
+      <c r="G26" s="92"/>
+      <c r="H26" s="92"/>
+      <c r="I26" s="92"/>
+      <c r="J26" s="92"/>
+      <c r="K26" s="92"/>
+      <c r="L26" s="92"/>
+      <c r="M26" s="92"/>
+      <c r="N26" s="92"/>
       <c r="O26" s="1"/>
     </row>
     <row r="27" spans="1:15" ht="29" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="76" t="s">
+      <c r="B27" s="82" t="s">
         <v>91</v>
       </c>
-      <c r="C27" s="82"/>
+      <c r="C27" s="80"/>
       <c r="D27" s="33">
         <v>10</v>
       </c>
@@ -11657,140 +11652,140 @@
     </row>
     <row r="28" spans="1:15" ht="24" customHeight="1">
       <c r="A28" s="1"/>
-      <c r="B28" s="94" t="s">
+      <c r="B28" s="88" t="s">
         <v>92</v>
       </c>
-      <c r="C28" s="95"/>
-      <c r="D28" s="95"/>
-      <c r="E28" s="95"/>
-      <c r="F28" s="95"/>
-      <c r="G28" s="95"/>
-      <c r="H28" s="95"/>
-      <c r="I28" s="95"/>
-      <c r="J28" s="95"/>
-      <c r="K28" s="95"/>
-      <c r="L28" s="95"/>
-      <c r="M28" s="95"/>
-      <c r="N28" s="95"/>
+      <c r="C28" s="89"/>
+      <c r="D28" s="89"/>
+      <c r="E28" s="89"/>
+      <c r="F28" s="89"/>
+      <c r="G28" s="89"/>
+      <c r="H28" s="89"/>
+      <c r="I28" s="89"/>
+      <c r="J28" s="89"/>
+      <c r="K28" s="89"/>
+      <c r="L28" s="89"/>
+      <c r="M28" s="89"/>
+      <c r="N28" s="89"/>
       <c r="O28" s="1"/>
     </row>
     <row r="29" spans="1:15" ht="23.15" customHeight="1">
       <c r="A29" s="1"/>
-      <c r="B29" s="93"/>
-      <c r="C29" s="93"/>
-      <c r="D29" s="93"/>
-      <c r="E29" s="93"/>
-      <c r="F29" s="93"/>
-      <c r="G29" s="93"/>
-      <c r="H29" s="93"/>
-      <c r="I29" s="93"/>
-      <c r="J29" s="93"/>
-      <c r="K29" s="93"/>
-      <c r="L29" s="93"/>
-      <c r="M29" s="93"/>
-      <c r="N29" s="93"/>
+      <c r="B29" s="87"/>
+      <c r="C29" s="87"/>
+      <c r="D29" s="87"/>
+      <c r="E29" s="87"/>
+      <c r="F29" s="87"/>
+      <c r="G29" s="87"/>
+      <c r="H29" s="87"/>
+      <c r="I29" s="87"/>
+      <c r="J29" s="87"/>
+      <c r="K29" s="87"/>
+      <c r="L29" s="87"/>
+      <c r="M29" s="87"/>
+      <c r="N29" s="87"/>
       <c r="O29" s="1"/>
     </row>
     <row r="30" spans="1:15" ht="31" customHeight="1">
       <c r="A30" s="1"/>
-      <c r="B30" s="96"/>
-      <c r="C30" s="96"/>
-      <c r="D30" s="96"/>
-      <c r="E30" s="96"/>
-      <c r="F30" s="96"/>
-      <c r="G30" s="96"/>
-      <c r="H30" s="96"/>
-      <c r="I30" s="96"/>
-      <c r="J30" s="96"/>
-      <c r="K30" s="96"/>
-      <c r="L30" s="96"/>
-      <c r="M30" s="96"/>
-      <c r="N30" s="96"/>
+      <c r="B30" s="90"/>
+      <c r="C30" s="90"/>
+      <c r="D30" s="90"/>
+      <c r="E30" s="90"/>
+      <c r="F30" s="90"/>
+      <c r="G30" s="90"/>
+      <c r="H30" s="90"/>
+      <c r="I30" s="90"/>
+      <c r="J30" s="90"/>
+      <c r="K30" s="90"/>
+      <c r="L30" s="90"/>
+      <c r="M30" s="90"/>
+      <c r="N30" s="90"/>
       <c r="O30" s="1"/>
     </row>
     <row r="31" spans="1:15" ht="23.15" customHeight="1">
       <c r="A31" s="1"/>
-      <c r="B31" s="93"/>
-      <c r="C31" s="93"/>
-      <c r="D31" s="93"/>
-      <c r="E31" s="93"/>
-      <c r="F31" s="93"/>
-      <c r="G31" s="93"/>
-      <c r="H31" s="93"/>
-      <c r="I31" s="93"/>
-      <c r="J31" s="93"/>
-      <c r="K31" s="93"/>
-      <c r="L31" s="93"/>
-      <c r="M31" s="93"/>
-      <c r="N31" s="93"/>
+      <c r="B31" s="87"/>
+      <c r="C31" s="87"/>
+      <c r="D31" s="87"/>
+      <c r="E31" s="87"/>
+      <c r="F31" s="87"/>
+      <c r="G31" s="87"/>
+      <c r="H31" s="87"/>
+      <c r="I31" s="87"/>
+      <c r="J31" s="87"/>
+      <c r="K31" s="87"/>
+      <c r="L31" s="87"/>
+      <c r="M31" s="87"/>
+      <c r="N31" s="87"/>
       <c r="O31" s="1"/>
     </row>
     <row r="32" spans="1:15" ht="23.15" customHeight="1">
       <c r="A32" s="1"/>
-      <c r="B32" s="93"/>
-      <c r="C32" s="93"/>
-      <c r="D32" s="93"/>
-      <c r="E32" s="93"/>
-      <c r="F32" s="93"/>
-      <c r="G32" s="93"/>
-      <c r="H32" s="93"/>
-      <c r="I32" s="93"/>
-      <c r="J32" s="93"/>
-      <c r="K32" s="93"/>
-      <c r="L32" s="93"/>
-      <c r="M32" s="93"/>
-      <c r="N32" s="93"/>
+      <c r="B32" s="87"/>
+      <c r="C32" s="87"/>
+      <c r="D32" s="87"/>
+      <c r="E32" s="87"/>
+      <c r="F32" s="87"/>
+      <c r="G32" s="87"/>
+      <c r="H32" s="87"/>
+      <c r="I32" s="87"/>
+      <c r="J32" s="87"/>
+      <c r="K32" s="87"/>
+      <c r="L32" s="87"/>
+      <c r="M32" s="87"/>
+      <c r="N32" s="87"/>
       <c r="O32" s="1"/>
     </row>
     <row r="33" spans="1:15" ht="23.15" customHeight="1">
       <c r="A33" s="1"/>
-      <c r="B33" s="93"/>
-      <c r="C33" s="93"/>
-      <c r="D33" s="93"/>
-      <c r="E33" s="93"/>
-      <c r="F33" s="93"/>
-      <c r="G33" s="93"/>
-      <c r="H33" s="93"/>
-      <c r="I33" s="93"/>
-      <c r="J33" s="93"/>
-      <c r="K33" s="93"/>
-      <c r="L33" s="93"/>
-      <c r="M33" s="93"/>
-      <c r="N33" s="93"/>
+      <c r="B33" s="87"/>
+      <c r="C33" s="87"/>
+      <c r="D33" s="87"/>
+      <c r="E33" s="87"/>
+      <c r="F33" s="87"/>
+      <c r="G33" s="87"/>
+      <c r="H33" s="87"/>
+      <c r="I33" s="87"/>
+      <c r="J33" s="87"/>
+      <c r="K33" s="87"/>
+      <c r="L33" s="87"/>
+      <c r="M33" s="87"/>
+      <c r="N33" s="87"/>
       <c r="O33" s="1"/>
     </row>
     <row r="34" spans="1:15" ht="23.15" customHeight="1">
       <c r="A34" s="1"/>
-      <c r="B34" s="93"/>
-      <c r="C34" s="93"/>
-      <c r="D34" s="93"/>
-      <c r="E34" s="93"/>
-      <c r="F34" s="93"/>
-      <c r="G34" s="93"/>
-      <c r="H34" s="93"/>
-      <c r="I34" s="93"/>
-      <c r="J34" s="93"/>
-      <c r="K34" s="93"/>
-      <c r="L34" s="93"/>
-      <c r="M34" s="93"/>
-      <c r="N34" s="93"/>
+      <c r="B34" s="87"/>
+      <c r="C34" s="87"/>
+      <c r="D34" s="87"/>
+      <c r="E34" s="87"/>
+      <c r="F34" s="87"/>
+      <c r="G34" s="87"/>
+      <c r="H34" s="87"/>
+      <c r="I34" s="87"/>
+      <c r="J34" s="87"/>
+      <c r="K34" s="87"/>
+      <c r="L34" s="87"/>
+      <c r="M34" s="87"/>
+      <c r="N34" s="87"/>
       <c r="O34" s="1"/>
     </row>
     <row r="35" spans="1:15" ht="23.15" customHeight="1">
       <c r="A35" s="1"/>
-      <c r="B35" s="93"/>
-      <c r="C35" s="93"/>
-      <c r="D35" s="93"/>
-      <c r="E35" s="93"/>
-      <c r="F35" s="93"/>
-      <c r="G35" s="93"/>
-      <c r="H35" s="93"/>
-      <c r="I35" s="93"/>
-      <c r="J35" s="93"/>
-      <c r="K35" s="93"/>
-      <c r="L35" s="93"/>
-      <c r="M35" s="93"/>
-      <c r="N35" s="93"/>
+      <c r="B35" s="87"/>
+      <c r="C35" s="87"/>
+      <c r="D35" s="87"/>
+      <c r="E35" s="87"/>
+      <c r="F35" s="87"/>
+      <c r="G35" s="87"/>
+      <c r="H35" s="87"/>
+      <c r="I35" s="87"/>
+      <c r="J35" s="87"/>
+      <c r="K35" s="87"/>
+      <c r="L35" s="87"/>
+      <c r="M35" s="87"/>
+      <c r="N35" s="87"/>
       <c r="O35" s="1"/>
     </row>
     <row r="36" spans="1:15" ht="23.15" customHeight="1">
@@ -11897,14 +11892,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="B33:N33"/>
-    <mergeCell ref="B34:N34"/>
-    <mergeCell ref="B35:N35"/>
-    <mergeCell ref="B28:N28"/>
-    <mergeCell ref="B29:N29"/>
-    <mergeCell ref="B30:N30"/>
-    <mergeCell ref="B31:N31"/>
-    <mergeCell ref="B32:N32"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B2:N2"/>
     <mergeCell ref="B3:N3"/>
@@ -11917,6 +11904,14 @@
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="F23:N24"/>
     <mergeCell ref="F26:N26"/>
+    <mergeCell ref="B33:N33"/>
+    <mergeCell ref="B34:N34"/>
+    <mergeCell ref="B35:N35"/>
+    <mergeCell ref="B28:N28"/>
+    <mergeCell ref="B29:N29"/>
+    <mergeCell ref="B30:N30"/>
+    <mergeCell ref="B31:N31"/>
+    <mergeCell ref="B32:N32"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11938,29 +11933,29 @@
   <sheetData>
     <row r="1" spans="1:22" ht="32" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="97" t="s">
+      <c r="B1" s="96" t="s">
         <v>93</v>
       </c>
-      <c r="C1" s="97"/>
-      <c r="D1" s="97"/>
-      <c r="E1" s="97"/>
-      <c r="F1" s="97"/>
-      <c r="G1" s="97"/>
-      <c r="H1" s="97"/>
-      <c r="I1" s="97"/>
-      <c r="J1" s="97"/>
-      <c r="K1" s="97"/>
-      <c r="L1" s="97"/>
-      <c r="M1" s="97"/>
-      <c r="N1" s="97"/>
-      <c r="O1" s="97"/>
-      <c r="P1" s="98"/>
-      <c r="Q1" s="98"/>
-      <c r="R1" s="98"/>
-      <c r="S1" s="98"/>
-      <c r="T1" s="98"/>
-      <c r="U1" s="98"/>
-      <c r="V1" s="98"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="96"/>
+      <c r="I1" s="96"/>
+      <c r="J1" s="96"/>
+      <c r="K1" s="96"/>
+      <c r="L1" s="96"/>
+      <c r="M1" s="96"/>
+      <c r="N1" s="96"/>
+      <c r="O1" s="96"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
     </row>
     <row r="2" spans="1:22" ht="22" customHeight="1">
       <c r="A2" s="1"/>
@@ -13631,29 +13626,29 @@
     </row>
     <row r="41" spans="1:22" ht="32" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="97" t="s">
+      <c r="B41" s="96" t="s">
         <v>94</v>
       </c>
-      <c r="C41" s="97"/>
-      <c r="D41" s="97"/>
-      <c r="E41" s="97"/>
-      <c r="F41" s="97"/>
-      <c r="G41" s="97"/>
-      <c r="H41" s="97"/>
-      <c r="I41" s="97"/>
-      <c r="J41" s="97"/>
-      <c r="K41" s="97"/>
-      <c r="L41" s="97"/>
-      <c r="M41" s="97"/>
-      <c r="N41" s="97"/>
-      <c r="O41" s="97"/>
-      <c r="P41" s="98"/>
-      <c r="Q41" s="98"/>
-      <c r="R41" s="98"/>
-      <c r="S41" s="98"/>
-      <c r="T41" s="98"/>
-      <c r="U41" s="98"/>
-      <c r="V41" s="98"/>
+      <c r="C41" s="96"/>
+      <c r="D41" s="96"/>
+      <c r="E41" s="96"/>
+      <c r="F41" s="96"/>
+      <c r="G41" s="96"/>
+      <c r="H41" s="96"/>
+      <c r="I41" s="96"/>
+      <c r="J41" s="96"/>
+      <c r="K41" s="96"/>
+      <c r="L41" s="96"/>
+      <c r="M41" s="96"/>
+      <c r="N41" s="96"/>
+      <c r="O41" s="96"/>
+      <c r="P41" s="97"/>
+      <c r="Q41" s="97"/>
+      <c r="R41" s="97"/>
+      <c r="S41" s="97"/>
+      <c r="T41" s="97"/>
+      <c r="U41" s="97"/>
+      <c r="V41" s="97"/>
     </row>
     <row r="42" spans="1:22" ht="22" customHeight="1">
       <c r="A42" s="1"/>
@@ -15285,29 +15280,29 @@
       <c r="V80" s="4"/>
     </row>
     <row r="81" spans="2:22" ht="32" customHeight="1">
-      <c r="B81" s="98" t="s">
+      <c r="B81" s="97" t="s">
         <v>95</v>
       </c>
-      <c r="C81" s="98"/>
-      <c r="D81" s="98"/>
-      <c r="E81" s="98"/>
-      <c r="F81" s="98"/>
-      <c r="G81" s="98"/>
-      <c r="H81" s="98"/>
-      <c r="I81" s="98"/>
-      <c r="J81" s="98"/>
-      <c r="K81" s="98"/>
-      <c r="L81" s="98"/>
-      <c r="M81" s="98"/>
-      <c r="N81" s="98"/>
-      <c r="O81" s="98"/>
-      <c r="P81" s="98"/>
-      <c r="Q81" s="98"/>
-      <c r="R81" s="98"/>
-      <c r="S81" s="98"/>
-      <c r="T81" s="98"/>
-      <c r="U81" s="98"/>
-      <c r="V81" s="98"/>
+      <c r="C81" s="97"/>
+      <c r="D81" s="97"/>
+      <c r="E81" s="97"/>
+      <c r="F81" s="97"/>
+      <c r="G81" s="97"/>
+      <c r="H81" s="97"/>
+      <c r="I81" s="97"/>
+      <c r="J81" s="97"/>
+      <c r="K81" s="97"/>
+      <c r="L81" s="97"/>
+      <c r="M81" s="97"/>
+      <c r="N81" s="97"/>
+      <c r="O81" s="97"/>
+      <c r="P81" s="97"/>
+      <c r="Q81" s="97"/>
+      <c r="R81" s="97"/>
+      <c r="S81" s="97"/>
+      <c r="T81" s="97"/>
+      <c r="U81" s="97"/>
+      <c r="V81" s="97"/>
     </row>
     <row r="82" spans="2:22" ht="22" customHeight="1">
       <c r="B82" s="4"/>
@@ -16938,29 +16933,29 @@
       <c r="V120" s="4"/>
     </row>
     <row r="121" spans="2:22" ht="32" customHeight="1">
-      <c r="B121" s="98" t="s">
+      <c r="B121" s="97" t="s">
         <v>96</v>
       </c>
-      <c r="C121" s="98"/>
-      <c r="D121" s="98"/>
-      <c r="E121" s="98"/>
-      <c r="F121" s="98"/>
-      <c r="G121" s="98"/>
-      <c r="H121" s="98"/>
-      <c r="I121" s="98"/>
-      <c r="J121" s="98"/>
-      <c r="K121" s="98"/>
-      <c r="L121" s="98"/>
-      <c r="M121" s="98"/>
-      <c r="N121" s="98"/>
-      <c r="O121" s="98"/>
-      <c r="P121" s="98"/>
-      <c r="Q121" s="98"/>
-      <c r="R121" s="98"/>
-      <c r="S121" s="98"/>
-      <c r="T121" s="98"/>
-      <c r="U121" s="98"/>
-      <c r="V121" s="98"/>
+      <c r="C121" s="97"/>
+      <c r="D121" s="97"/>
+      <c r="E121" s="97"/>
+      <c r="F121" s="97"/>
+      <c r="G121" s="97"/>
+      <c r="H121" s="97"/>
+      <c r="I121" s="97"/>
+      <c r="J121" s="97"/>
+      <c r="K121" s="97"/>
+      <c r="L121" s="97"/>
+      <c r="M121" s="97"/>
+      <c r="N121" s="97"/>
+      <c r="O121" s="97"/>
+      <c r="P121" s="97"/>
+      <c r="Q121" s="97"/>
+      <c r="R121" s="97"/>
+      <c r="S121" s="97"/>
+      <c r="T121" s="97"/>
+      <c r="U121" s="97"/>
+      <c r="V121" s="97"/>
     </row>
     <row r="122" spans="2:22" ht="22" customHeight="1">
       <c r="B122" s="4"/>
@@ -18852,29 +18847,29 @@
       <c r="V157" s="4"/>
     </row>
     <row r="161" spans="2:22" ht="32" customHeight="1">
-      <c r="B161" s="99" t="s">
+      <c r="B161" s="98" t="s">
         <v>97</v>
       </c>
-      <c r="C161" s="99"/>
-      <c r="D161" s="99"/>
-      <c r="E161" s="99"/>
-      <c r="F161" s="99"/>
-      <c r="G161" s="99"/>
-      <c r="H161" s="99"/>
-      <c r="I161" s="99"/>
-      <c r="J161" s="99"/>
-      <c r="K161" s="99"/>
-      <c r="L161" s="99"/>
-      <c r="M161" s="99"/>
-      <c r="N161" s="99"/>
-      <c r="O161" s="99"/>
-      <c r="P161" s="99"/>
-      <c r="Q161" s="99"/>
-      <c r="R161" s="99"/>
-      <c r="S161" s="99"/>
-      <c r="T161" s="99"/>
-      <c r="U161" s="99"/>
-      <c r="V161" s="99"/>
+      <c r="C161" s="98"/>
+      <c r="D161" s="98"/>
+      <c r="E161" s="98"/>
+      <c r="F161" s="98"/>
+      <c r="G161" s="98"/>
+      <c r="H161" s="98"/>
+      <c r="I161" s="98"/>
+      <c r="J161" s="98"/>
+      <c r="K161" s="98"/>
+      <c r="L161" s="98"/>
+      <c r="M161" s="98"/>
+      <c r="N161" s="98"/>
+      <c r="O161" s="98"/>
+      <c r="P161" s="98"/>
+      <c r="Q161" s="98"/>
+      <c r="R161" s="98"/>
+      <c r="S161" s="98"/>
+      <c r="T161" s="98"/>
+      <c r="U161" s="98"/>
+      <c r="V161" s="98"/>
     </row>
     <row r="164" spans="2:22" ht="44" customHeight="1">
       <c r="B164" s="63" t="s">

</xml_diff>

<commit_message>
RX damper and other fixes
</commit_message>
<xml_diff>
--- a/docs/damping_curve_RAx0.xlsx
+++ b/docs/damping_curve_RAx0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mods\unpacked\un1corn_qlourie_astral_r\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\un1corn\.codex\visualizations\2026\09\05\01a07025-ed7a-7f60-89f7-3275b6531400\damping-rx-sync-20261026\native\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E71426E-0C2C-43A5-9E07-AAA127F4B1D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ACEAC72-8851-44CF-AEBC-70E45295771A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalog" sheetId="8" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="99">
   <si>
     <t>Valving</t>
   </si>
@@ -366,6 +366,10 @@
   </si>
   <si>
     <t>Calculator</t>
+  </si>
+  <si>
+    <t>Type-A</t>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1880,11 +1884,11 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1899,13 +1903,13 @@
     <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1920,28 +1924,28 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="8" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="8" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="8" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1950,7 +1954,7 @@
     <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2082,17 +2086,56 @@
     <xf numFmtId="0" fontId="82" fillId="71" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="26" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="34" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="35" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="28" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="24" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="43" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="44" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="45" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="46" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="47" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2106,35 +2149,8 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="32" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="33" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="23" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="24" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="26" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="28" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="28" fillId="17" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -2142,32 +2158,17 @@
     <xf numFmtId="2" fontId="29" fillId="18" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="57" fillId="46" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="23" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="47" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="43" fillId="32" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="34" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="33" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="35" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="54" fillId="43" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="44" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="45" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="59" fillId="48" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -6199,19 +6200,14 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="10287000" cy="5143500"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart">
@@ -6234,25 +6230,20 @@
       </a:graphic>
     </xdr:graphicFrame>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="10287000" cy="5143500"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart">
@@ -6275,25 +6266,20 @@
       </a:graphic>
     </xdr:graphicFrame>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="10287000" cy="5143500"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart">
@@ -6316,25 +6302,20 @@
       </a:graphic>
     </xdr:graphicFrame>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="10287000" cy="5143500"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart">
@@ -6357,7 +6338,7 @@
       </a:graphic>
     </xdr:graphicFrame>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -6582,14 +6563,14 @@
     </row>
     <row r="2" spans="1:8" ht="35" customHeight="1">
       <c r="A2" s="6"/>
-      <c r="B2" s="72" t="s">
+      <c r="B2" s="85" t="s">
         <v>84</v>
       </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
+      <c r="C2" s="86"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
       <c r="H2" s="6"/>
     </row>
     <row r="3" spans="1:8" ht="25" customHeight="1">
@@ -6640,7 +6621,7 @@
     </row>
     <row r="6" spans="1:8" ht="31" customHeight="1">
       <c r="A6" s="6"/>
-      <c r="B6" s="74" t="s">
+      <c r="B6" s="87" t="s">
         <v>81</v>
       </c>
       <c r="C6" s="6"/>
@@ -6660,7 +6641,7 @@
     </row>
     <row r="7" spans="1:8" ht="31" customHeight="1">
       <c r="A7" s="6"/>
-      <c r="B7" s="74"/>
+      <c r="B7" s="87"/>
       <c r="C7" s="6"/>
       <c r="D7" s="19" t="s">
         <v>77</v>
@@ -6792,40 +6773,40 @@
       <c r="A15" s="6"/>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
-      <c r="D15" s="71"/>
-      <c r="E15" s="71"/>
-      <c r="F15" s="71"/>
-      <c r="G15" s="71"/>
+      <c r="D15" s="84"/>
+      <c r="E15" s="84"/>
+      <c r="F15" s="84"/>
+      <c r="G15" s="84"/>
       <c r="H15" s="6"/>
     </row>
     <row r="16" spans="1:8" ht="22" customHeight="1">
       <c r="A16" s="6"/>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
-      <c r="D16" s="71"/>
-      <c r="E16" s="71"/>
-      <c r="F16" s="71"/>
-      <c r="G16" s="71"/>
+      <c r="D16" s="84"/>
+      <c r="E16" s="84"/>
+      <c r="F16" s="84"/>
+      <c r="G16" s="84"/>
       <c r="H16" s="6"/>
     </row>
     <row r="17" spans="1:8" ht="22" customHeight="1">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
-      <c r="D17" s="69"/>
-      <c r="E17" s="71"/>
-      <c r="F17" s="71"/>
-      <c r="G17" s="71"/>
+      <c r="D17" s="68"/>
+      <c r="E17" s="84"/>
+      <c r="F17" s="84"/>
+      <c r="G17" s="84"/>
       <c r="H17" s="6"/>
     </row>
     <row r="18" spans="1:8" ht="22" customHeight="1">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
-      <c r="D18" s="71"/>
-      <c r="E18" s="71"/>
-      <c r="F18" s="71"/>
-      <c r="G18" s="71"/>
+      <c r="D18" s="84"/>
+      <c r="E18" s="84"/>
+      <c r="F18" s="84"/>
+      <c r="G18" s="84"/>
       <c r="H18" s="6"/>
     </row>
     <row r="19" spans="1:8" ht="25" customHeight="1">
@@ -6907,20 +6888,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
       <c r="N2" s="24"/>
       <c r="O2" s="1"/>
     </row>
@@ -6947,18 +6928,18 @@
         <v>0</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>1</v>
+        <v>98</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
+      <c r="E4" s="88"/>
+      <c r="F4" s="88"/>
+      <c r="G4" s="88"/>
+      <c r="H4" s="88"/>
+      <c r="I4" s="88"/>
+      <c r="J4" s="88"/>
+      <c r="K4" s="88"/>
+      <c r="L4" s="88"/>
+      <c r="M4" s="88"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -6989,13 +6970,13 @@
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
-      <c r="F6" s="83" t="s">
+      <c r="F6" s="73" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="84"/>
-      <c r="H6" s="84"/>
-      <c r="I6" s="84"/>
-      <c r="J6" s="84"/>
+      <c r="G6" s="72"/>
+      <c r="H6" s="72"/>
+      <c r="I6" s="72"/>
+      <c r="J6" s="72"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
@@ -7033,16 +7014,16 @@
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
-      <c r="F8" s="82" t="s">
+      <c r="F8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="79"/>
-      <c r="H8" s="79"/>
-      <c r="I8" s="85">
+      <c r="G8" s="76"/>
+      <c r="H8" s="76"/>
+      <c r="I8" s="89">
         <f>IF(C18="OK",Samples!F165*MIN(C10,Samples!G165)+Samples!I165*MAX(0,C10-Samples!G165)+Samples!J165*MAX(0,C10-Samples!K165),"检查输入")</f>
         <v>1736.47</v>
       </c>
-      <c r="J8" s="86"/>
+      <c r="J8" s="90"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
@@ -7080,16 +7061,16 @@
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="82" t="s">
+      <c r="F10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="79"/>
-      <c r="H10" s="79"/>
-      <c r="I10" s="85">
+      <c r="G10" s="76"/>
+      <c r="H10" s="76"/>
+      <c r="I10" s="89">
         <f>IF(C18="OK",Samples!M165*MIN(C10,Samples!N165)+Samples!P165*MAX(0,C10-Samples!N165),"检查输入")</f>
         <v>1519.2</v>
       </c>
-      <c r="J10" s="86"/>
+      <c r="J10" s="90"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
@@ -7141,13 +7122,13 @@
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="F13" s="83" t="s">
+      <c r="F13" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="G13" s="84"/>
-      <c r="H13" s="84"/>
-      <c r="I13" s="84"/>
-      <c r="J13" s="84"/>
+      <c r="G13" s="72"/>
+      <c r="H13" s="72"/>
+      <c r="I13" s="72"/>
+      <c r="J13" s="72"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
@@ -7165,11 +7146,11 @@
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
-      <c r="F14" s="77" t="s">
+      <c r="F14" s="91" t="s">
         <v>10</v>
       </c>
-      <c r="G14" s="78"/>
-      <c r="H14" s="78"/>
+      <c r="G14" s="75"/>
+      <c r="H14" s="75"/>
       <c r="I14" s="34">
         <f>Samples!F165</f>
         <v>3650</v>
@@ -7194,11 +7175,11 @@
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
-      <c r="F15" s="79" t="s">
+      <c r="F15" s="76" t="s">
         <v>26</v>
       </c>
-      <c r="G15" s="80"/>
-      <c r="H15" s="80"/>
+      <c r="G15" s="67"/>
+      <c r="H15" s="67"/>
       <c r="I15" s="35">
         <f>Samples!I165</f>
         <v>3431</v>
@@ -7218,11 +7199,11 @@
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="81" t="s">
+      <c r="F16" s="74" t="s">
         <v>48</v>
       </c>
-      <c r="G16" s="78"/>
-      <c r="H16" s="78"/>
+      <c r="G16" s="75"/>
+      <c r="H16" s="75"/>
       <c r="I16" s="34">
         <f>Samples!J165</f>
         <v>1750</v>
@@ -7242,11 +7223,11 @@
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
-      <c r="F17" s="82" t="s">
+      <c r="F17" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G17" s="80"/>
-      <c r="H17" s="80"/>
+      <c r="G17" s="67"/>
+      <c r="H17" s="67"/>
       <c r="I17" s="35">
         <f>Samples!L165</f>
         <v>5181</v>
@@ -7288,11 +7269,11 @@
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
-      <c r="F19" s="77" t="s">
+      <c r="F19" s="91" t="s">
         <v>15</v>
       </c>
-      <c r="G19" s="78"/>
-      <c r="H19" s="78"/>
+      <c r="G19" s="75"/>
+      <c r="H19" s="75"/>
       <c r="I19" s="34">
         <f>Samples!M165</f>
         <v>3600</v>
@@ -7312,11 +7293,11 @@
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
-      <c r="F20" s="79" t="s">
+      <c r="F20" s="76" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="80"/>
-      <c r="H20" s="80"/>
+      <c r="G20" s="67"/>
+      <c r="H20" s="67"/>
       <c r="I20" s="35">
         <f>Samples!P165</f>
         <v>3096</v>
@@ -7353,11 +7334,11 @@
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="81" t="s">
+      <c r="F22" s="74" t="s">
         <v>44</v>
       </c>
-      <c r="G22" s="78"/>
-      <c r="H22" s="78"/>
+      <c r="G22" s="75"/>
+      <c r="H22" s="75"/>
       <c r="I22" s="37">
         <f>Samples!G165</f>
         <v>0.08</v>
@@ -7377,11 +7358,11 @@
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="82" t="s">
+      <c r="F23" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G23" s="80"/>
-      <c r="H23" s="80"/>
+      <c r="G23" s="67"/>
+      <c r="H23" s="67"/>
       <c r="I23" s="38">
         <f>Samples!K165</f>
         <v>0.35</v>
@@ -7401,11 +7382,11 @@
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="77" t="s">
+      <c r="F24" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="G24" s="78"/>
-      <c r="H24" s="78"/>
+      <c r="G24" s="75"/>
+      <c r="H24" s="75"/>
       <c r="I24" s="37">
         <f>Samples!N165</f>
         <v>0.25</v>
@@ -7455,20 +7436,20 @@
     </row>
     <row r="27" spans="1:15" ht="23.15" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="75" t="s">
+      <c r="B27" s="92" t="s">
         <v>87</v>
       </c>
-      <c r="C27" s="76"/>
-      <c r="D27" s="76"/>
-      <c r="E27" s="76"/>
-      <c r="F27" s="76"/>
-      <c r="G27" s="76"/>
-      <c r="H27" s="76"/>
-      <c r="I27" s="76"/>
-      <c r="J27" s="76"/>
-      <c r="K27" s="76"/>
-      <c r="L27" s="76"/>
-      <c r="M27" s="76"/>
+      <c r="C27" s="93"/>
+      <c r="D27" s="93"/>
+      <c r="E27" s="93"/>
+      <c r="F27" s="93"/>
+      <c r="G27" s="93"/>
+      <c r="H27" s="93"/>
+      <c r="I27" s="93"/>
+      <c r="J27" s="93"/>
+      <c r="K27" s="93"/>
+      <c r="L27" s="93"/>
+      <c r="M27" s="93"/>
       <c r="N27" s="1"/>
       <c r="O27" s="1"/>
     </row>
@@ -7729,6 +7710,17 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B27:M27"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="F24:H24"/>
+    <mergeCell ref="F13:J13"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="F17:H17"/>
     <mergeCell ref="B2:M2"/>
     <mergeCell ref="E4:M4"/>
     <mergeCell ref="F6:J6"/>
@@ -7736,17 +7728,6 @@
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="I10:J10"/>
-    <mergeCell ref="F13:J13"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="F16:H16"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="B27:M27"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="F24:H24"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <dataValidations count="5">
@@ -7803,20 +7784,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="68" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
       <c r="N2" s="24"/>
       <c r="O2" s="1"/>
     </row>
@@ -7846,15 +7827,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
+      <c r="E4" s="88"/>
+      <c r="F4" s="88"/>
+      <c r="G4" s="88"/>
+      <c r="H4" s="88"/>
+      <c r="I4" s="88"/>
+      <c r="J4" s="88"/>
+      <c r="K4" s="88"/>
+      <c r="L4" s="88"/>
+      <c r="M4" s="88"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -7884,15 +7865,15 @@
         <v>-10</v>
       </c>
       <c r="D6" s="1"/>
-      <c r="E6" s="69"/>
-      <c r="F6" s="69"/>
-      <c r="G6" s="69"/>
-      <c r="H6" s="69"/>
-      <c r="I6" s="69"/>
-      <c r="J6" s="69"/>
-      <c r="K6" s="69"/>
-      <c r="L6" s="69"/>
-      <c r="M6" s="69"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="68"/>
+      <c r="I6" s="68"/>
+      <c r="J6" s="68"/>
+      <c r="K6" s="68"/>
+      <c r="L6" s="68"/>
+      <c r="M6" s="68"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -8476,18 +8457,18 @@
     </row>
     <row r="41" spans="1:15" ht="23.15" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="70"/>
-      <c r="C41" s="70"/>
-      <c r="D41" s="70"/>
-      <c r="E41" s="70"/>
-      <c r="F41" s="70"/>
-      <c r="G41" s="70"/>
-      <c r="H41" s="70"/>
-      <c r="I41" s="70"/>
-      <c r="J41" s="70"/>
-      <c r="K41" s="70"/>
-      <c r="L41" s="70"/>
-      <c r="M41" s="70"/>
+      <c r="B41" s="94"/>
+      <c r="C41" s="94"/>
+      <c r="D41" s="94"/>
+      <c r="E41" s="94"/>
+      <c r="F41" s="94"/>
+      <c r="G41" s="94"/>
+      <c r="H41" s="94"/>
+      <c r="I41" s="94"/>
+      <c r="J41" s="94"/>
+      <c r="K41" s="94"/>
+      <c r="L41" s="94"/>
+      <c r="M41" s="94"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -8561,20 +8542,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="68" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
       <c r="N2" s="24"/>
       <c r="O2" s="1"/>
     </row>
@@ -8604,15 +8585,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
+      <c r="E4" s="88"/>
+      <c r="F4" s="88"/>
+      <c r="G4" s="88"/>
+      <c r="H4" s="88"/>
+      <c r="I4" s="88"/>
+      <c r="J4" s="88"/>
+      <c r="K4" s="88"/>
+      <c r="L4" s="88"/>
+      <c r="M4" s="88"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -8642,15 +8623,15 @@
         <v>-12</v>
       </c>
       <c r="D6" s="1"/>
-      <c r="E6" s="69"/>
-      <c r="F6" s="69"/>
-      <c r="G6" s="69"/>
-      <c r="H6" s="69"/>
-      <c r="I6" s="69"/>
-      <c r="J6" s="69"/>
-      <c r="K6" s="69"/>
-      <c r="L6" s="69"/>
-      <c r="M6" s="69"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="68"/>
+      <c r="I6" s="68"/>
+      <c r="J6" s="68"/>
+      <c r="K6" s="68"/>
+      <c r="L6" s="68"/>
+      <c r="M6" s="68"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -9234,18 +9215,18 @@
     </row>
     <row r="41" spans="1:15" ht="23.15" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="70"/>
-      <c r="C41" s="70"/>
-      <c r="D41" s="70"/>
-      <c r="E41" s="70"/>
-      <c r="F41" s="70"/>
-      <c r="G41" s="70"/>
-      <c r="H41" s="70"/>
-      <c r="I41" s="70"/>
-      <c r="J41" s="70"/>
-      <c r="K41" s="70"/>
-      <c r="L41" s="70"/>
-      <c r="M41" s="70"/>
+      <c r="B41" s="94"/>
+      <c r="C41" s="94"/>
+      <c r="D41" s="94"/>
+      <c r="E41" s="94"/>
+      <c r="F41" s="94"/>
+      <c r="G41" s="94"/>
+      <c r="H41" s="94"/>
+      <c r="I41" s="94"/>
+      <c r="J41" s="94"/>
+      <c r="K41" s="94"/>
+      <c r="L41" s="94"/>
+      <c r="M41" s="94"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -9319,20 +9300,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="68" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
       <c r="N2" s="24"/>
       <c r="O2" s="1"/>
     </row>
@@ -9362,15 +9343,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
+      <c r="E4" s="88"/>
+      <c r="F4" s="88"/>
+      <c r="G4" s="88"/>
+      <c r="H4" s="88"/>
+      <c r="I4" s="88"/>
+      <c r="J4" s="88"/>
+      <c r="K4" s="88"/>
+      <c r="L4" s="88"/>
+      <c r="M4" s="88"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -9393,18 +9374,18 @@
     </row>
     <row r="6" spans="1:15" ht="28" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="69"/>
-      <c r="C6" s="69"/>
-      <c r="D6" s="69"/>
-      <c r="E6" s="69"/>
-      <c r="F6" s="69"/>
-      <c r="G6" s="69"/>
-      <c r="H6" s="69"/>
-      <c r="I6" s="69"/>
-      <c r="J6" s="69"/>
-      <c r="K6" s="69"/>
-      <c r="L6" s="69"/>
-      <c r="M6" s="69"/>
+      <c r="B6" s="68"/>
+      <c r="C6" s="68"/>
+      <c r="D6" s="68"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="68"/>
+      <c r="I6" s="68"/>
+      <c r="J6" s="68"/>
+      <c r="K6" s="68"/>
+      <c r="L6" s="68"/>
+      <c r="M6" s="68"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -9988,18 +9969,18 @@
     </row>
     <row r="41" spans="1:15" ht="23.15" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="70"/>
-      <c r="C41" s="70"/>
-      <c r="D41" s="70"/>
-      <c r="E41" s="70"/>
-      <c r="F41" s="70"/>
-      <c r="G41" s="70"/>
-      <c r="H41" s="70"/>
-      <c r="I41" s="70"/>
-      <c r="J41" s="70"/>
-      <c r="K41" s="70"/>
-      <c r="L41" s="70"/>
-      <c r="M41" s="70"/>
+      <c r="B41" s="94"/>
+      <c r="C41" s="94"/>
+      <c r="D41" s="94"/>
+      <c r="E41" s="94"/>
+      <c r="F41" s="94"/>
+      <c r="G41" s="94"/>
+      <c r="H41" s="94"/>
+      <c r="I41" s="94"/>
+      <c r="J41" s="94"/>
+      <c r="K41" s="94"/>
+      <c r="L41" s="94"/>
+      <c r="M41" s="94"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -10069,20 +10050,20 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="68" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
       <c r="N2" s="24"/>
       <c r="O2" s="1"/>
     </row>
@@ -10112,15 +10093,15 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
+      <c r="E4" s="88"/>
+      <c r="F4" s="88"/>
+      <c r="G4" s="88"/>
+      <c r="H4" s="88"/>
+      <c r="I4" s="88"/>
+      <c r="J4" s="88"/>
+      <c r="K4" s="88"/>
+      <c r="L4" s="88"/>
+      <c r="M4" s="88"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -10143,18 +10124,18 @@
     </row>
     <row r="6" spans="1:15" ht="28" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="69"/>
-      <c r="C6" s="69"/>
-      <c r="D6" s="69"/>
-      <c r="E6" s="69"/>
-      <c r="F6" s="69"/>
-      <c r="G6" s="69"/>
-      <c r="H6" s="69"/>
-      <c r="I6" s="69"/>
-      <c r="J6" s="69"/>
-      <c r="K6" s="69"/>
-      <c r="L6" s="69"/>
-      <c r="M6" s="69"/>
+      <c r="B6" s="68"/>
+      <c r="C6" s="68"/>
+      <c r="D6" s="68"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="68"/>
+      <c r="I6" s="68"/>
+      <c r="J6" s="68"/>
+      <c r="K6" s="68"/>
+      <c r="L6" s="68"/>
+      <c r="M6" s="68"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
@@ -10738,18 +10719,18 @@
     </row>
     <row r="41" spans="1:15" ht="23.15" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="70"/>
-      <c r="C41" s="70"/>
-      <c r="D41" s="70"/>
-      <c r="E41" s="70"/>
-      <c r="F41" s="70"/>
-      <c r="G41" s="70"/>
-      <c r="H41" s="70"/>
-      <c r="I41" s="70"/>
-      <c r="J41" s="70"/>
-      <c r="K41" s="70"/>
-      <c r="L41" s="70"/>
-      <c r="M41" s="70"/>
+      <c r="B41" s="94"/>
+      <c r="C41" s="94"/>
+      <c r="D41" s="94"/>
+      <c r="E41" s="94"/>
+      <c r="F41" s="94"/>
+      <c r="G41" s="94"/>
+      <c r="H41" s="94"/>
+      <c r="I41" s="94"/>
+      <c r="J41" s="94"/>
+      <c r="K41" s="94"/>
+      <c r="L41" s="94"/>
+      <c r="M41" s="94"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -10823,40 +10804,40 @@
     </row>
     <row r="2" spans="1:15" ht="35" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="68" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
-      <c r="N2" s="67"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
       <c r="O2" s="1"/>
     </row>
     <row r="3" spans="1:15" ht="24" customHeight="1">
       <c r="A3" s="1"/>
-      <c r="B3" s="91" t="s">
+      <c r="B3" s="70" t="s">
         <v>87</v>
       </c>
-      <c r="C3" s="92"/>
-      <c r="D3" s="92"/>
-      <c r="E3" s="92"/>
-      <c r="F3" s="92"/>
-      <c r="G3" s="92"/>
-      <c r="H3" s="92"/>
-      <c r="I3" s="92"/>
-      <c r="J3" s="92"/>
-      <c r="K3" s="92"/>
-      <c r="L3" s="92"/>
-      <c r="M3" s="92"/>
-      <c r="N3" s="92"/>
+      <c r="C3" s="71"/>
+      <c r="D3" s="71"/>
+      <c r="E3" s="71"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="71"/>
+      <c r="I3" s="71"/>
+      <c r="J3" s="71"/>
+      <c r="K3" s="71"/>
+      <c r="L3" s="71"/>
+      <c r="M3" s="71"/>
+      <c r="N3" s="71"/>
       <c r="O3" s="1"/>
     </row>
     <row r="4" spans="1:15" ht="28" customHeight="1">
@@ -10880,21 +10861,21 @@
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
-      <c r="D5" s="84" t="s">
+      <c r="D5" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="84"/>
-      <c r="F5" s="84"/>
-      <c r="G5" s="84"/>
-      <c r="H5" s="84"/>
+      <c r="E5" s="72"/>
+      <c r="F5" s="72"/>
+      <c r="G5" s="72"/>
+      <c r="H5" s="72"/>
       <c r="I5" s="1"/>
-      <c r="J5" s="84" t="s">
+      <c r="J5" s="72" t="s">
         <v>4</v>
       </c>
-      <c r="K5" s="84"/>
-      <c r="L5" s="84"/>
-      <c r="M5" s="84"/>
-      <c r="N5" s="84"/>
+      <c r="K5" s="72"/>
+      <c r="L5" s="72"/>
+      <c r="M5" s="72"/>
+      <c r="N5" s="72"/>
       <c r="O5" s="1"/>
     </row>
     <row r="6" spans="1:15" ht="30" customHeight="1">
@@ -11470,21 +11451,21 @@
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="42">
-        <v>0.68</v>
+        <v>0.74</v>
       </c>
       <c r="K19" s="37">
         <f>(J19+L19)/2</f>
-        <v>0.65</v>
+        <v>0.71</v>
       </c>
       <c r="L19" s="42">
-        <v>0.62</v>
+        <v>0.68</v>
       </c>
       <c r="M19" s="37">
         <f>(L19+N19)/2</f>
-        <v>0.59000000000000008</v>
+        <v>0.65</v>
       </c>
       <c r="N19" s="42">
-        <v>0.56000000000000005</v>
+        <v>0.62</v>
       </c>
       <c r="O19" s="1"/>
     </row>
@@ -11524,73 +11505,73 @@
     </row>
     <row r="22" spans="1:15" ht="32" customHeight="1">
       <c r="A22" s="1"/>
-      <c r="B22" s="83" t="s">
+      <c r="B22" s="73" t="s">
         <v>52</v>
       </c>
-      <c r="C22" s="84"/>
-      <c r="D22" s="84"/>
-      <c r="E22" s="84"/>
-      <c r="F22" s="84"/>
-      <c r="G22" s="84"/>
-      <c r="H22" s="84"/>
-      <c r="I22" s="84"/>
-      <c r="J22" s="84"/>
-      <c r="K22" s="84"/>
-      <c r="L22" s="84"/>
-      <c r="M22" s="84"/>
-      <c r="N22" s="84"/>
+      <c r="C22" s="72"/>
+      <c r="D22" s="72"/>
+      <c r="E22" s="72"/>
+      <c r="F22" s="72"/>
+      <c r="G22" s="72"/>
+      <c r="H22" s="72"/>
+      <c r="I22" s="72"/>
+      <c r="J22" s="72"/>
+      <c r="K22" s="72"/>
+      <c r="L22" s="72"/>
+      <c r="M22" s="72"/>
+      <c r="N22" s="72"/>
       <c r="O22" s="1"/>
     </row>
     <row r="23" spans="1:15" ht="29" customHeight="1">
       <c r="A23" s="1"/>
-      <c r="B23" s="81" t="s">
+      <c r="B23" s="74" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="78"/>
+      <c r="C23" s="75"/>
       <c r="D23" s="31">
         <v>24</v>
       </c>
       <c r="E23" s="1"/>
-      <c r="F23" s="93" t="s">
+      <c r="F23" s="77" t="s">
         <v>88</v>
       </c>
-      <c r="G23" s="94"/>
-      <c r="H23" s="94"/>
-      <c r="I23" s="94"/>
-      <c r="J23" s="94"/>
-      <c r="K23" s="94"/>
-      <c r="L23" s="94"/>
-      <c r="M23" s="94"/>
-      <c r="N23" s="94"/>
+      <c r="G23" s="78"/>
+      <c r="H23" s="78"/>
+      <c r="I23" s="78"/>
+      <c r="J23" s="78"/>
+      <c r="K23" s="78"/>
+      <c r="L23" s="78"/>
+      <c r="M23" s="78"/>
+      <c r="N23" s="78"/>
       <c r="O23" s="1"/>
     </row>
     <row r="24" spans="1:15" ht="29" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="82" t="s">
+      <c r="B24" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C24" s="80"/>
+      <c r="C24" s="67"/>
       <c r="D24" s="33">
         <v>20</v>
       </c>
       <c r="E24" s="1"/>
-      <c r="F24" s="94"/>
-      <c r="G24" s="94"/>
-      <c r="H24" s="94"/>
-      <c r="I24" s="94"/>
-      <c r="J24" s="94"/>
-      <c r="K24" s="94"/>
-      <c r="L24" s="94"/>
-      <c r="M24" s="94"/>
-      <c r="N24" s="94"/>
+      <c r="F24" s="78"/>
+      <c r="G24" s="78"/>
+      <c r="H24" s="78"/>
+      <c r="I24" s="78"/>
+      <c r="J24" s="78"/>
+      <c r="K24" s="78"/>
+      <c r="L24" s="78"/>
+      <c r="M24" s="78"/>
+      <c r="N24" s="78"/>
       <c r="O24" s="1"/>
     </row>
     <row r="25" spans="1:15" ht="29" customHeight="1">
       <c r="A25" s="1"/>
-      <c r="B25" s="81" t="s">
+      <c r="B25" s="74" t="s">
         <v>60</v>
       </c>
-      <c r="C25" s="78"/>
+      <c r="C25" s="75"/>
       <c r="D25" s="31">
         <v>40</v>
       </c>
@@ -11608,33 +11589,33 @@
     </row>
     <row r="26" spans="1:15" ht="29" customHeight="1">
       <c r="A26" s="1"/>
-      <c r="B26" s="79" t="s">
+      <c r="B26" s="76" t="s">
         <v>54</v>
       </c>
-      <c r="C26" s="80"/>
+      <c r="C26" s="67"/>
       <c r="D26" s="33">
         <v>60</v>
       </c>
       <c r="E26" s="1"/>
-      <c r="F26" s="95" t="s">
+      <c r="F26" s="79" t="s">
         <v>90</v>
       </c>
-      <c r="G26" s="92"/>
-      <c r="H26" s="92"/>
-      <c r="I26" s="92"/>
-      <c r="J26" s="92"/>
-      <c r="K26" s="92"/>
-      <c r="L26" s="92"/>
-      <c r="M26" s="92"/>
-      <c r="N26" s="92"/>
+      <c r="G26" s="71"/>
+      <c r="H26" s="71"/>
+      <c r="I26" s="71"/>
+      <c r="J26" s="71"/>
+      <c r="K26" s="71"/>
+      <c r="L26" s="71"/>
+      <c r="M26" s="71"/>
+      <c r="N26" s="71"/>
       <c r="O26" s="1"/>
     </row>
     <row r="27" spans="1:15" ht="29" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="82" t="s">
+      <c r="B27" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C27" s="80"/>
+      <c r="C27" s="67"/>
       <c r="D27" s="33">
         <v>10</v>
       </c>
@@ -11652,140 +11633,140 @@
     </row>
     <row r="28" spans="1:15" ht="24" customHeight="1">
       <c r="A28" s="1"/>
-      <c r="B28" s="88" t="s">
+      <c r="B28" s="81" t="s">
         <v>92</v>
       </c>
-      <c r="C28" s="89"/>
-      <c r="D28" s="89"/>
-      <c r="E28" s="89"/>
-      <c r="F28" s="89"/>
-      <c r="G28" s="89"/>
-      <c r="H28" s="89"/>
-      <c r="I28" s="89"/>
-      <c r="J28" s="89"/>
-      <c r="K28" s="89"/>
-      <c r="L28" s="89"/>
-      <c r="M28" s="89"/>
-      <c r="N28" s="89"/>
+      <c r="C28" s="82"/>
+      <c r="D28" s="82"/>
+      <c r="E28" s="82"/>
+      <c r="F28" s="82"/>
+      <c r="G28" s="82"/>
+      <c r="H28" s="82"/>
+      <c r="I28" s="82"/>
+      <c r="J28" s="82"/>
+      <c r="K28" s="82"/>
+      <c r="L28" s="82"/>
+      <c r="M28" s="82"/>
+      <c r="N28" s="82"/>
       <c r="O28" s="1"/>
     </row>
     <row r="29" spans="1:15" ht="23.15" customHeight="1">
       <c r="A29" s="1"/>
-      <c r="B29" s="87"/>
-      <c r="C29" s="87"/>
-      <c r="D29" s="87"/>
-      <c r="E29" s="87"/>
-      <c r="F29" s="87"/>
-      <c r="G29" s="87"/>
-      <c r="H29" s="87"/>
-      <c r="I29" s="87"/>
-      <c r="J29" s="87"/>
-      <c r="K29" s="87"/>
-      <c r="L29" s="87"/>
-      <c r="M29" s="87"/>
-      <c r="N29" s="87"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="80"/>
+      <c r="F29" s="80"/>
+      <c r="G29" s="80"/>
+      <c r="H29" s="80"/>
+      <c r="I29" s="80"/>
+      <c r="J29" s="80"/>
+      <c r="K29" s="80"/>
+      <c r="L29" s="80"/>
+      <c r="M29" s="80"/>
+      <c r="N29" s="80"/>
       <c r="O29" s="1"/>
     </row>
     <row r="30" spans="1:15" ht="31" customHeight="1">
       <c r="A30" s="1"/>
-      <c r="B30" s="90"/>
-      <c r="C30" s="90"/>
-      <c r="D30" s="90"/>
-      <c r="E30" s="90"/>
-      <c r="F30" s="90"/>
-      <c r="G30" s="90"/>
-      <c r="H30" s="90"/>
-      <c r="I30" s="90"/>
-      <c r="J30" s="90"/>
-      <c r="K30" s="90"/>
-      <c r="L30" s="90"/>
-      <c r="M30" s="90"/>
-      <c r="N30" s="90"/>
+      <c r="B30" s="83"/>
+      <c r="C30" s="83"/>
+      <c r="D30" s="83"/>
+      <c r="E30" s="83"/>
+      <c r="F30" s="83"/>
+      <c r="G30" s="83"/>
+      <c r="H30" s="83"/>
+      <c r="I30" s="83"/>
+      <c r="J30" s="83"/>
+      <c r="K30" s="83"/>
+      <c r="L30" s="83"/>
+      <c r="M30" s="83"/>
+      <c r="N30" s="83"/>
       <c r="O30" s="1"/>
     </row>
     <row r="31" spans="1:15" ht="23.15" customHeight="1">
       <c r="A31" s="1"/>
-      <c r="B31" s="87"/>
-      <c r="C31" s="87"/>
-      <c r="D31" s="87"/>
-      <c r="E31" s="87"/>
-      <c r="F31" s="87"/>
-      <c r="G31" s="87"/>
-      <c r="H31" s="87"/>
-      <c r="I31" s="87"/>
-      <c r="J31" s="87"/>
-      <c r="K31" s="87"/>
-      <c r="L31" s="87"/>
-      <c r="M31" s="87"/>
-      <c r="N31" s="87"/>
+      <c r="B31" s="80"/>
+      <c r="C31" s="80"/>
+      <c r="D31" s="80"/>
+      <c r="E31" s="80"/>
+      <c r="F31" s="80"/>
+      <c r="G31" s="80"/>
+      <c r="H31" s="80"/>
+      <c r="I31" s="80"/>
+      <c r="J31" s="80"/>
+      <c r="K31" s="80"/>
+      <c r="L31" s="80"/>
+      <c r="M31" s="80"/>
+      <c r="N31" s="80"/>
       <c r="O31" s="1"/>
     </row>
     <row r="32" spans="1:15" ht="23.15" customHeight="1">
       <c r="A32" s="1"/>
-      <c r="B32" s="87"/>
-      <c r="C32" s="87"/>
-      <c r="D32" s="87"/>
-      <c r="E32" s="87"/>
-      <c r="F32" s="87"/>
-      <c r="G32" s="87"/>
-      <c r="H32" s="87"/>
-      <c r="I32" s="87"/>
-      <c r="J32" s="87"/>
-      <c r="K32" s="87"/>
-      <c r="L32" s="87"/>
-      <c r="M32" s="87"/>
-      <c r="N32" s="87"/>
+      <c r="B32" s="80"/>
+      <c r="C32" s="80"/>
+      <c r="D32" s="80"/>
+      <c r="E32" s="80"/>
+      <c r="F32" s="80"/>
+      <c r="G32" s="80"/>
+      <c r="H32" s="80"/>
+      <c r="I32" s="80"/>
+      <c r="J32" s="80"/>
+      <c r="K32" s="80"/>
+      <c r="L32" s="80"/>
+      <c r="M32" s="80"/>
+      <c r="N32" s="80"/>
       <c r="O32" s="1"/>
     </row>
     <row r="33" spans="1:15" ht="23.15" customHeight="1">
       <c r="A33" s="1"/>
-      <c r="B33" s="87"/>
-      <c r="C33" s="87"/>
-      <c r="D33" s="87"/>
-      <c r="E33" s="87"/>
-      <c r="F33" s="87"/>
-      <c r="G33" s="87"/>
-      <c r="H33" s="87"/>
-      <c r="I33" s="87"/>
-      <c r="J33" s="87"/>
-      <c r="K33" s="87"/>
-      <c r="L33" s="87"/>
-      <c r="M33" s="87"/>
-      <c r="N33" s="87"/>
+      <c r="B33" s="80"/>
+      <c r="C33" s="80"/>
+      <c r="D33" s="80"/>
+      <c r="E33" s="80"/>
+      <c r="F33" s="80"/>
+      <c r="G33" s="80"/>
+      <c r="H33" s="80"/>
+      <c r="I33" s="80"/>
+      <c r="J33" s="80"/>
+      <c r="K33" s="80"/>
+      <c r="L33" s="80"/>
+      <c r="M33" s="80"/>
+      <c r="N33" s="80"/>
       <c r="O33" s="1"/>
     </row>
     <row r="34" spans="1:15" ht="23.15" customHeight="1">
       <c r="A34" s="1"/>
-      <c r="B34" s="87"/>
-      <c r="C34" s="87"/>
-      <c r="D34" s="87"/>
-      <c r="E34" s="87"/>
-      <c r="F34" s="87"/>
-      <c r="G34" s="87"/>
-      <c r="H34" s="87"/>
-      <c r="I34" s="87"/>
-      <c r="J34" s="87"/>
-      <c r="K34" s="87"/>
-      <c r="L34" s="87"/>
-      <c r="M34" s="87"/>
-      <c r="N34" s="87"/>
+      <c r="B34" s="80"/>
+      <c r="C34" s="80"/>
+      <c r="D34" s="80"/>
+      <c r="E34" s="80"/>
+      <c r="F34" s="80"/>
+      <c r="G34" s="80"/>
+      <c r="H34" s="80"/>
+      <c r="I34" s="80"/>
+      <c r="J34" s="80"/>
+      <c r="K34" s="80"/>
+      <c r="L34" s="80"/>
+      <c r="M34" s="80"/>
+      <c r="N34" s="80"/>
       <c r="O34" s="1"/>
     </row>
     <row r="35" spans="1:15" ht="23.15" customHeight="1">
       <c r="A35" s="1"/>
-      <c r="B35" s="87"/>
-      <c r="C35" s="87"/>
-      <c r="D35" s="87"/>
-      <c r="E35" s="87"/>
-      <c r="F35" s="87"/>
-      <c r="G35" s="87"/>
-      <c r="H35" s="87"/>
-      <c r="I35" s="87"/>
-      <c r="J35" s="87"/>
-      <c r="K35" s="87"/>
-      <c r="L35" s="87"/>
-      <c r="M35" s="87"/>
-      <c r="N35" s="87"/>
+      <c r="B35" s="80"/>
+      <c r="C35" s="80"/>
+      <c r="D35" s="80"/>
+      <c r="E35" s="80"/>
+      <c r="F35" s="80"/>
+      <c r="G35" s="80"/>
+      <c r="H35" s="80"/>
+      <c r="I35" s="80"/>
+      <c r="J35" s="80"/>
+      <c r="K35" s="80"/>
+      <c r="L35" s="80"/>
+      <c r="M35" s="80"/>
+      <c r="N35" s="80"/>
       <c r="O35" s="1"/>
     </row>
     <row r="36" spans="1:15" ht="23.15" customHeight="1">
@@ -11892,6 +11873,14 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B33:N33"/>
+    <mergeCell ref="B34:N34"/>
+    <mergeCell ref="B35:N35"/>
+    <mergeCell ref="B28:N28"/>
+    <mergeCell ref="B29:N29"/>
+    <mergeCell ref="B30:N30"/>
+    <mergeCell ref="B31:N31"/>
+    <mergeCell ref="B32:N32"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B2:N2"/>
     <mergeCell ref="B3:N3"/>
@@ -11904,14 +11893,6 @@
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="F23:N24"/>
     <mergeCell ref="F26:N26"/>
-    <mergeCell ref="B33:N33"/>
-    <mergeCell ref="B34:N34"/>
-    <mergeCell ref="B35:N35"/>
-    <mergeCell ref="B28:N28"/>
-    <mergeCell ref="B29:N29"/>
-    <mergeCell ref="B30:N30"/>
-    <mergeCell ref="B31:N31"/>
-    <mergeCell ref="B32:N32"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11933,29 +11914,29 @@
   <sheetData>
     <row r="1" spans="1:22" ht="32" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="96" t="s">
+      <c r="B1" s="95" t="s">
         <v>93</v>
       </c>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
-      <c r="L1" s="96"/>
-      <c r="M1" s="96"/>
-      <c r="N1" s="96"/>
-      <c r="O1" s="96"/>
-      <c r="P1" s="97"/>
-      <c r="Q1" s="97"/>
-      <c r="R1" s="97"/>
-      <c r="S1" s="97"/>
-      <c r="T1" s="97"/>
-      <c r="U1" s="97"/>
-      <c r="V1" s="97"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="95"/>
+      <c r="I1" s="95"/>
+      <c r="J1" s="95"/>
+      <c r="K1" s="95"/>
+      <c r="L1" s="95"/>
+      <c r="M1" s="95"/>
+      <c r="N1" s="95"/>
+      <c r="O1" s="95"/>
+      <c r="P1" s="96"/>
+      <c r="Q1" s="96"/>
+      <c r="R1" s="96"/>
+      <c r="S1" s="96"/>
+      <c r="T1" s="96"/>
+      <c r="U1" s="96"/>
+      <c r="V1" s="96"/>
     </row>
     <row r="2" spans="1:22" ht="22" customHeight="1">
       <c r="A2" s="1"/>
@@ -13626,29 +13607,29 @@
     </row>
     <row r="41" spans="1:22" ht="32" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="96" t="s">
+      <c r="B41" s="95" t="s">
         <v>94</v>
       </c>
-      <c r="C41" s="96"/>
-      <c r="D41" s="96"/>
-      <c r="E41" s="96"/>
-      <c r="F41" s="96"/>
-      <c r="G41" s="96"/>
-      <c r="H41" s="96"/>
-      <c r="I41" s="96"/>
-      <c r="J41" s="96"/>
-      <c r="K41" s="96"/>
-      <c r="L41" s="96"/>
-      <c r="M41" s="96"/>
-      <c r="N41" s="96"/>
-      <c r="O41" s="96"/>
-      <c r="P41" s="97"/>
-      <c r="Q41" s="97"/>
-      <c r="R41" s="97"/>
-      <c r="S41" s="97"/>
-      <c r="T41" s="97"/>
-      <c r="U41" s="97"/>
-      <c r="V41" s="97"/>
+      <c r="C41" s="95"/>
+      <c r="D41" s="95"/>
+      <c r="E41" s="95"/>
+      <c r="F41" s="95"/>
+      <c r="G41" s="95"/>
+      <c r="H41" s="95"/>
+      <c r="I41" s="95"/>
+      <c r="J41" s="95"/>
+      <c r="K41" s="95"/>
+      <c r="L41" s="95"/>
+      <c r="M41" s="95"/>
+      <c r="N41" s="95"/>
+      <c r="O41" s="95"/>
+      <c r="P41" s="96"/>
+      <c r="Q41" s="96"/>
+      <c r="R41" s="96"/>
+      <c r="S41" s="96"/>
+      <c r="T41" s="96"/>
+      <c r="U41" s="96"/>
+      <c r="V41" s="96"/>
     </row>
     <row r="42" spans="1:22" ht="22" customHeight="1">
       <c r="A42" s="1"/>
@@ -15280,29 +15261,29 @@
       <c r="V80" s="4"/>
     </row>
     <row r="81" spans="2:22" ht="32" customHeight="1">
-      <c r="B81" s="97" t="s">
+      <c r="B81" s="96" t="s">
         <v>95</v>
       </c>
-      <c r="C81" s="97"/>
-      <c r="D81" s="97"/>
-      <c r="E81" s="97"/>
-      <c r="F81" s="97"/>
-      <c r="G81" s="97"/>
-      <c r="H81" s="97"/>
-      <c r="I81" s="97"/>
-      <c r="J81" s="97"/>
-      <c r="K81" s="97"/>
-      <c r="L81" s="97"/>
-      <c r="M81" s="97"/>
-      <c r="N81" s="97"/>
-      <c r="O81" s="97"/>
-      <c r="P81" s="97"/>
-      <c r="Q81" s="97"/>
-      <c r="R81" s="97"/>
-      <c r="S81" s="97"/>
-      <c r="T81" s="97"/>
-      <c r="U81" s="97"/>
-      <c r="V81" s="97"/>
+      <c r="C81" s="96"/>
+      <c r="D81" s="96"/>
+      <c r="E81" s="96"/>
+      <c r="F81" s="96"/>
+      <c r="G81" s="96"/>
+      <c r="H81" s="96"/>
+      <c r="I81" s="96"/>
+      <c r="J81" s="96"/>
+      <c r="K81" s="96"/>
+      <c r="L81" s="96"/>
+      <c r="M81" s="96"/>
+      <c r="N81" s="96"/>
+      <c r="O81" s="96"/>
+      <c r="P81" s="96"/>
+      <c r="Q81" s="96"/>
+      <c r="R81" s="96"/>
+      <c r="S81" s="96"/>
+      <c r="T81" s="96"/>
+      <c r="U81" s="96"/>
+      <c r="V81" s="96"/>
     </row>
     <row r="82" spans="2:22" ht="22" customHeight="1">
       <c r="B82" s="4"/>
@@ -16933,29 +16914,29 @@
       <c r="V120" s="4"/>
     </row>
     <row r="121" spans="2:22" ht="32" customHeight="1">
-      <c r="B121" s="97" t="s">
+      <c r="B121" s="96" t="s">
         <v>96</v>
       </c>
-      <c r="C121" s="97"/>
-      <c r="D121" s="97"/>
-      <c r="E121" s="97"/>
-      <c r="F121" s="97"/>
-      <c r="G121" s="97"/>
-      <c r="H121" s="97"/>
-      <c r="I121" s="97"/>
-      <c r="J121" s="97"/>
-      <c r="K121" s="97"/>
-      <c r="L121" s="97"/>
-      <c r="M121" s="97"/>
-      <c r="N121" s="97"/>
-      <c r="O121" s="97"/>
-      <c r="P121" s="97"/>
-      <c r="Q121" s="97"/>
-      <c r="R121" s="97"/>
-      <c r="S121" s="97"/>
-      <c r="T121" s="97"/>
-      <c r="U121" s="97"/>
-      <c r="V121" s="97"/>
+      <c r="C121" s="96"/>
+      <c r="D121" s="96"/>
+      <c r="E121" s="96"/>
+      <c r="F121" s="96"/>
+      <c r="G121" s="96"/>
+      <c r="H121" s="96"/>
+      <c r="I121" s="96"/>
+      <c r="J121" s="96"/>
+      <c r="K121" s="96"/>
+      <c r="L121" s="96"/>
+      <c r="M121" s="96"/>
+      <c r="N121" s="96"/>
+      <c r="O121" s="96"/>
+      <c r="P121" s="96"/>
+      <c r="Q121" s="96"/>
+      <c r="R121" s="96"/>
+      <c r="S121" s="96"/>
+      <c r="T121" s="96"/>
+      <c r="U121" s="96"/>
+      <c r="V121" s="96"/>
     </row>
     <row r="122" spans="2:22" ht="22" customHeight="1">
       <c r="B122" s="4"/>
@@ -18847,29 +18828,29 @@
       <c r="V157" s="4"/>
     </row>
     <row r="161" spans="2:22" ht="32" customHeight="1">
-      <c r="B161" s="98" t="s">
+      <c r="B161" s="97" t="s">
         <v>97</v>
       </c>
-      <c r="C161" s="98"/>
-      <c r="D161" s="98"/>
-      <c r="E161" s="98"/>
-      <c r="F161" s="98"/>
-      <c r="G161" s="98"/>
-      <c r="H161" s="98"/>
-      <c r="I161" s="98"/>
-      <c r="J161" s="98"/>
-      <c r="K161" s="98"/>
-      <c r="L161" s="98"/>
-      <c r="M161" s="98"/>
-      <c r="N161" s="98"/>
-      <c r="O161" s="98"/>
-      <c r="P161" s="98"/>
-      <c r="Q161" s="98"/>
-      <c r="R161" s="98"/>
-      <c r="S161" s="98"/>
-      <c r="T161" s="98"/>
-      <c r="U161" s="98"/>
-      <c r="V161" s="98"/>
+      <c r="C161" s="97"/>
+      <c r="D161" s="97"/>
+      <c r="E161" s="97"/>
+      <c r="F161" s="97"/>
+      <c r="G161" s="97"/>
+      <c r="H161" s="97"/>
+      <c r="I161" s="97"/>
+      <c r="J161" s="97"/>
+      <c r="K161" s="97"/>
+      <c r="L161" s="97"/>
+      <c r="M161" s="97"/>
+      <c r="N161" s="97"/>
+      <c r="O161" s="97"/>
+      <c r="P161" s="97"/>
+      <c r="Q161" s="97"/>
+      <c r="R161" s="97"/>
+      <c r="S161" s="97"/>
+      <c r="T161" s="97"/>
+      <c r="U161" s="97"/>
+      <c r="V161" s="97"/>
     </row>
     <row r="164" spans="2:22" ht="44" customHeight="1">
       <c r="B164" s="63" t="s">

</xml_diff>